<commit_message>
feat(domain): add finite traveling merchant
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R60111b380267418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R6a27e7296de042bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="R6b7a5fd81eae4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rc20bed3139294257"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rc5ad47eb35b74aa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rd838a33182c74c11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R22aa57da08ce4879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R6c298670c1f0401d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R393d1d5127384c51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rf51648398bb4464d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="Rd72bb9835e6d4828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd01debd64970435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rf3ef459499a44a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Re7045e8d597c45c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rde47cc7ee03248f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R031103caeb564c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Re1d96fe4f09049cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Rb0143fd37b894269"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R6fa18e1edfd845ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R58f8617f78a64ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R21b57539f1934398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R1e3875c703f94a0e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -136,7 +136,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -184,6 +184,9 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -16940,10 +16943,10 @@
   <x:cols>
     <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -17085,60 +17088,60 @@
       <x:c r="A10" s="20" t="str">
         <x:v>MerchantStartingCash</x:v>
       </x:c>
-      <x:c r="B10" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B10" s="20" t="n">
+        <x:v>10000</x:v>
       </x:c>
       <x:c r="C10" s="20" t="str">
         <x:v>Gold</x:v>
       </x:c>
       <x:c r="D10" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E10" s="20" t="str">
-        <x:v>Vốn khởi điểm</x:v>
+        <x:v>Vốn khởi điểm để mô phỏng Merchant hữu hạn; cần cân bằng sau.</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="20" t="str">
         <x:v>MerchantCarryingCapacity</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B11" s="20" t="n">
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C11" s="20" t="str">
         <x:v>đơn vị vật phẩm</x:v>
       </x:c>
       <x:c r="D11" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E11" s="20" t="str">
-        <x:v>Sức chứa hàng hóa</x:v>
+        <x:v>Sức chứa hiện tại trong MerchantConfig; cần cân bằng sau.</x:v>
       </x:c>
       <x:c r="F11" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="20" t="str">
         <x:v>MerchantRouteCycleMinutes</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B12" s="20" t="n">
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C12" s="20" t="str">
         <x:v>phút in-game</x:v>
       </x:c>
       <x:c r="D12" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E12" s="20" t="str">
-        <x:v>Chu kỳ tuyến đường</x:v>
+        <x:v>Chu kỳ tuyến prototype để mô phỏng tuyến lưu động; cần cân bằng sau.</x:v>
       </x:c>
       <x:c r="F12" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -17165,80 +17168,148 @@
       <x:c r="A14" s="20" t="str">
         <x:v>MerchantBankruptcyCreditLimit</x:v>
       </x:c>
-      <x:c r="B14" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B14" s="20" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
         <x:v>Gold</x:v>
       </x:c>
       <x:c r="D14" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E14" s="20" t="str">
-        <x:v>Ngưỡng vốn âm trước phá sản</x:v>
+        <x:v>Merchant không vay; hoạt động với vốn hữu hạn.</x:v>
       </x:c>
       <x:c r="F14" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="20" t="str">
         <x:v>MerchantReplacementDelayMinutes</x:v>
       </x:c>
-      <x:c r="B15" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B15" s="20" t="n">
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C15" s="20" t="str">
         <x:v>phút in-game</x:v>
       </x:c>
       <x:c r="D15" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E15" s="20" t="str">
-        <x:v>Thời gian chờ thương nhân thay thế</x:v>
+        <x:v>Độ trễ đến của Merchant mới sau phá sản; cần cân bằng sau.</x:v>
       </x:c>
       <x:c r="F15" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="20" t="str">
         <x:v>MerchantMaximumWaitMinutes</x:v>
       </x:c>
-      <x:c r="B16" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B16" s="20" t="n">
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C16" s="20" t="str">
         <x:v>phút in-game</x:v>
       </x:c>
       <x:c r="D16" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>Thời gian chờ bán tối đa</x:v>
+        <x:v>Bảo đảm thời gian chờ hữu hạn khi tích hợp đánh thức Trainer.</x:v>
       </x:c>
       <x:c r="F16" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="20" t="str">
         <x:v>MerchantDiscountLotSizeThreshold</x:v>
       </x:c>
-      <x:c r="B17" s="20" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="B17" s="20" t="n">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C17" s="20" t="str">
         <x:v>đơn vị vật phẩm</x:v>
       </x:c>
       <x:c r="D17" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E17" s="20" t="str">
-        <x:v>Mốc lô cho spread theo khối lượng</x:v>
+        <x:v>Mốc lô làm spread tăng đơn điệu từ 5% lên 10%; giả định vì GDD chưa chốt chiều biến thiên.</x:v>
       </x:c>
       <x:c r="F17" s="20" t="str">
-        <x:v>docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+        <x:v>src/Game.Domain/Supply/Merchant.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>MerchantOperatingCostPerTrip</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>Gold/chặng</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>Chi phí mỗi chặng; dùng để mô phỏng và có thể gây phá sản.</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>src/Game.Domain/Supply/Merchant.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>MerchantSpreadLotDirection</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>Tăng theo lô</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>Quy tắc</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>Spread tăng theo quy mô lô; xác nhận lại khi playtest.</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>src/Game.Domain/Supply/Merchant.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>MerchantSpreadLotDirection</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Tăng theo lô</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>Quy tắc</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Spread tăng theo quy mô lô; xác nhận lại khi playtest.</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>src/Game.Domain/Supply/Merchant.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(domain): model workshop recipes and consumable stalls
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,17 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re9a09921f5cd4166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rc6996f8569574957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="R73877466ab5d457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rd00d12ecdb2345d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R2c78f141e64b479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="R537217dc102c49a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R69f06a9ae3c3485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R55ee0bb22c2e48a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R05c5279cc4e94caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R235a6d1d659f4ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R59d10a0dbb3e4d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Recddc9060dcb4af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R489745139da34290"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="R36861b422c4c41be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R0169ff10dfa94061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R7129a7dcc1724c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rdb507c7800094be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Rd73524bd9ee34af9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R15c96cea78c24fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rdf14d986773b43e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rce618d431d9a44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R43c4af3554df4d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R7d9c5672b50e4d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R22337f3ad2a24e60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -101,12 +103,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -136,7 +143,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -189,6 +196,14 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -450,11 +465,11 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="A10" s="32" t="str">
         <x:v>Sheet</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
-        <x:v>Nội dung</x:v>
+      <x:c r="B10" s="32" t="str">
+        <x:v>Contents</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -462,7 +477,7 @@
         <x:v>Parameters</x:v>
       </x:c>
       <x:c r="B11" s="4" t="str">
-        <x:v>Tham số của GDD 13, giữ nguyên nguồn và trạng thái</x:v>
+        <x:v>GDD balance parameters and sources</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -470,7 +485,7 @@
         <x:v>Domain Config</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>Giá trị hiện đang chạy trong SimConfig, phân biệt với GDD</x:v>
+        <x:v>Runtime defaults, separately labeled from GDD</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -478,47 +493,55 @@
         <x:v>Buildings / Backlog</x:v>
       </x:c>
       <x:c r="B13" s="4" t="str">
-        <x:v>Danh mục mô phỏng và câu hỏi/tham số chưa được định lượng</x:v>
+        <x:v>Building roles and open questions</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Material Catalog</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>30 nguyên liệu theo stable ID; sản phẩm, đơn vị, trạng thái và nguồn</x:v>
+      <x:c r="A14" s="4" t="str">
+        <x:v>Material / Product Catalog</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Stable material and product IDs</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>Recipe Inputs / Recipe Outputs</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>Đầu vào, đầu ra và định mức TBD theo công thức</x:v>
+      <x:c r="A15" s="4" t="str">
+        <x:v>Recipe Inputs / Outputs</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>75 inputs and 73 outputs, values labeled Prototype</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
+      <x:c r="A16" s="4" t="str">
         <x:v>Merchant</x:v>
       </x:c>
-      <x:c r="B16" t="str">
-        <x:v>Spread, thuế và tham số vận hành</x:v>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Cash, capacity, routes, spreads, and replacement drivers</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
+      <x:c r="A17" s="4" t="str">
         <x:v>Production Controls</x:v>
       </x:c>
-      <x:c r="B17" t="str">
-        <x:v>Mục tiêu tồn kho, định mức, thời gian và công suất</x:v>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Job timing, costs, producer capacity, and Refinery yield</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>Domain Config</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Tham số runtime hiện tại và ánh xạ mới cho supply chain</x:v>
+      <x:c r="A18" s="4" t="str">
+        <x:v>Equipment Workshops</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Three equipment slot groups from GDD 05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>Stalls</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Six shop-to-producer mappings from GDD 02/12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3997,6 +4020,7 @@
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -4037,6 +4061,9 @@
       <x:c r="G4" s="26" t="str">
         <x:v>Nguồn</x:v>
       </x:c>
+      <x:c r="H4" s="31" t="str">
+        <x:v>Effect metadata</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="25" t="str">
@@ -4060,6 +4087,7 @@
       <x:c r="G5" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H5" s="4" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="25" t="str">
@@ -4083,6 +4111,7 @@
       <x:c r="G6" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H6" s="4" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="25" t="str">
@@ -4106,6 +4135,7 @@
       <x:c r="G7" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H7" s="4" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="25" t="str">
@@ -4129,6 +4159,7 @@
       <x:c r="G8" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H8" s="4" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="25" t="str">
@@ -4152,6 +4183,7 @@
       <x:c r="G9" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H9" s="4" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="25" t="str">
@@ -4175,6 +4207,7 @@
       <x:c r="G10" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H10" s="4" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="25" t="str">
@@ -4198,6 +4231,7 @@
       <x:c r="G11" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H11" s="4" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="25" t="str">
@@ -4221,6 +4255,7 @@
       <x:c r="G12" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H12" s="4" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="25" t="str">
@@ -4244,6 +4279,7 @@
       <x:c r="G13" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H13" s="4" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="25" t="str">
@@ -4267,6 +4303,7 @@
       <x:c r="G14" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H14" s="4" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="25" t="str">
@@ -4290,6 +4327,7 @@
       <x:c r="G15" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H15" s="4" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="25" t="str">
@@ -4313,6 +4351,7 @@
       <x:c r="G16" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H16" s="4" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="25" t="str">
@@ -4336,6 +4375,7 @@
       <x:c r="G17" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H17" s="4" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="25" t="str">
@@ -4359,6 +4399,7 @@
       <x:c r="G18" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H18" s="4" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="25" t="str">
@@ -4382,6 +4423,9 @@
       <x:c r="G19" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>TemporaryMonsterStatBuff; chi tiết chỉ số TBD</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="25" t="str">
@@ -4405,6 +4449,7 @@
       <x:c r="G20" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H20" s="4" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="25" t="str">
@@ -4428,6 +4473,7 @@
       <x:c r="G21" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H21" s="4" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="25" t="str">
@@ -4451,6 +4497,7 @@
       <x:c r="G22" s="25" t="str">
         <x:v>docs/designs/05_Itemization_Gear_System.md; docs/designs/12_Item_Catalog.md §2</x:v>
       </x:c>
+      <x:c r="H22" s="4" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="25" t="str">
@@ -4474,6 +4521,7 @@
       <x:c r="G23" s="25" t="str">
         <x:v>docs/designs/05_Itemization_Gear_System.md; docs/designs/12_Item_Catalog.md §2</x:v>
       </x:c>
+      <x:c r="H23" s="4" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="25" t="str">
@@ -4497,6 +4545,7 @@
       <x:c r="G24" s="25" t="str">
         <x:v>docs/designs/05_Itemization_Gear_System.md; docs/designs/12_Item_Catalog.md §2</x:v>
       </x:c>
+      <x:c r="H24" s="4" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="25" t="str">
@@ -4520,6 +4569,7 @@
       <x:c r="G25" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H25" s="4" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="25" t="str">
@@ -4543,6 +4593,7 @@
       <x:c r="G26" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H26" s="4" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="25" t="str">
@@ -4566,6 +4617,7 @@
       <x:c r="G27" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H27" s="4" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="25" t="str">
@@ -4589,6 +4641,7 @@
       <x:c r="G28" s="25" t="str">
         <x:v>docs/designs/12_Item_Catalog.md §1-2</x:v>
       </x:c>
+      <x:c r="H28" s="4" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="25" t="str">
@@ -4612,6 +4665,7 @@
       <x:c r="G29" s="25" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H29" s="4" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
@@ -4635,6 +4689,7 @@
       <x:c r="G30" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H30" s="4" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
@@ -4658,6 +4713,7 @@
       <x:c r="G31" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H31" s="4" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
@@ -4681,6 +4737,7 @@
       <x:c r="G32" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H32" s="4" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="26" t="str">
@@ -4704,6 +4761,7 @@
       <x:c r="G33" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H33" s="4" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="24" t="str">
@@ -4727,6 +4785,7 @@
       <x:c r="G34" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H34" s="4" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="24" t="str">
@@ -4750,6 +4809,7 @@
       <x:c r="G35" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H35" s="4" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="24" t="str">
@@ -4773,6 +4833,7 @@
       <x:c r="G36" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H36" s="4" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="24" t="str">
@@ -4796,6 +4857,7 @@
       <x:c r="G37" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H37" s="4" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="24" t="str">
@@ -4819,6 +4881,7 @@
       <x:c r="G38" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H38" s="4" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="24" t="str">
@@ -4842,6 +4905,7 @@
       <x:c r="G39" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H39" s="4" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="24" t="str">
@@ -4865,6 +4929,7 @@
       <x:c r="G40" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H40" s="4" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="24" t="str">
@@ -4888,6 +4953,7 @@
       <x:c r="G41" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H41" s="4" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="24" t="str">
@@ -4911,6 +4977,7 @@
       <x:c r="G42" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H42" s="4" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="24" t="str">
@@ -4934,6 +5001,7 @@
       <x:c r="G43" t="str">
         <x:v>GDD 12 §2; GDD 02 §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
+      <x:c r="H43" s="4" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="24"/>
@@ -5240,6 +5308,293 @@
       </x:c>
       <x:c r="F60" t="str">
         <x:v>src/Game.Domain/Production/ProductionController.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Equipment workshop groups</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>The three slot groups defined by GDD 05.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="31" t="str">
+        <x:v>Producer ID</x:v>
+      </x:c>
+      <x:c r="B4" s="31" t="str">
+        <x:v>Nhóm slot</x:v>
+      </x:c>
+      <x:c r="C4" s="31" t="str">
+        <x:v>Số slot</x:v>
+      </x:c>
+      <x:c r="D4" s="31" t="str">
+        <x:v>Đơn vị chủ</x:v>
+      </x:c>
+      <x:c r="E4" s="31" t="str">
+        <x:v>Sản phẩm catalog</x:v>
+      </x:c>
+      <x:c r="F4" s="31" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="G4" s="31" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>monster_forge</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>Monster combat</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>mỗi Monster</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>monster_gear</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="str">
+        <x:v>docs/designs/05_Itemization_Gear_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>trainer_textile_workshop</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Trainer utility</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>mỗi Trainer</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>trainer_utility_gear</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>docs/designs/05_Itemization_Gear_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>aura_jeweler</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Aura</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>mỗi Trainer</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>aura_gear</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>docs/designs/05_Itemization_Gear_System.md §1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="56" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="60" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Consumable stall mapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Stalls sell produced stock. Service recovery consumes no inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="31" t="str">
+        <x:v>Shop ID</x:v>
+      </x:c>
+      <x:c r="B4" s="31" t="str">
+        <x:v>Producer ID</x:v>
+      </x:c>
+      <x:c r="C4" s="31" t="str">
+        <x:v>Product IDs</x:v>
+      </x:c>
+      <x:c r="D4" s="31" t="str">
+        <x:v>Hành vi</x:v>
+      </x:c>
+      <x:c r="E4" s="31" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="F4" s="31" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>potion; vaccine; tranquilizer</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Bán tồn kho đã sản xuất; hồi HP không tiêu thụ sản phẩm</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0, §1.4; docs/designs/12_Item_Catalog.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>food_drink; reward_cake</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Bán tồn kho đã sản xuất</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0; docs/designs/12_Item_Catalog.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>bar</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>bar</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>liquor</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Bán tồn kho đã sản xuất</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0; docs/designs/12_Item_Catalog.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="4" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>raincoat; gas_mask; capture_ball; trap; tactics_book</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Bán tồn kho đã sản xuất</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0; docs/designs/12_Item_Catalog.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>inn</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>inn</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>overclock_coffee</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Bán tồn kho đã sản xuất; ngủ nghỉ không tiêu thụ sản phẩm</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>docs/designs/12_Item_Catalog.md §1; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="4" t="str">
+        <x:v>general_store</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>soda_factory</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>monster_buff_bottle</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Nhà Máy Nước Ngọt sản xuất; Tiệm Tạp hóa bán</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0-1.1; docs/designs/12_Item_Catalog.md §1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17913,6 +18268,441 @@
         <x:v>GDD 02 §1.0; docs/designs/12_Item_Catalog.md; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="27" t="str">
+        <x:v>hospital_potion</x:v>
+      </x:c>
+      <x:c r="B65" s="27" t="str">
+        <x:v>Chế Thuốc từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C65" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D65" s="27" t="str">
+        <x:v>herb_tier_1</x:v>
+      </x:c>
+      <x:c r="E65" s="27" t="str">
+        <x:v>Thảo dược Tier 1</x:v>
+      </x:c>
+      <x:c r="F65" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G65" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H65" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I65" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="27" t="str">
+        <x:v>hospital_vaccine</x:v>
+      </x:c>
+      <x:c r="B66" s="27" t="str">
+        <x:v>Chế Vắc-xin từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C66" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D66" s="27" t="str">
+        <x:v>herb_tier_1</x:v>
+      </x:c>
+      <x:c r="E66" s="27" t="str">
+        <x:v>Thảo dược Tier 1</x:v>
+      </x:c>
+      <x:c r="F66" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G66" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H66" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I66" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="27" t="str">
+        <x:v>hospital_tranquilizer</x:v>
+      </x:c>
+      <x:c r="B67" s="27" t="str">
+        <x:v>Chế Thuốc An Thần từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C67" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D67" s="27" t="str">
+        <x:v>herb_tier_1</x:v>
+      </x:c>
+      <x:c r="E67" s="27" t="str">
+        <x:v>Thảo dược Tier 1</x:v>
+      </x:c>
+      <x:c r="F67" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G67" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H67" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I67" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="27" t="str">
+        <x:v>restaurant_food_drink</x:v>
+      </x:c>
+      <x:c r="B68" s="27" t="str">
+        <x:v>Chế Đồ ăn, nước uống từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C68" s="27" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D68" s="27" t="str">
+        <x:v>food_tier_1</x:v>
+      </x:c>
+      <x:c r="E68" s="27" t="str">
+        <x:v>Thực phẩm Tier 1</x:v>
+      </x:c>
+      <x:c r="F68" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G68" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H68" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I68" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="27" t="str">
+        <x:v>restaurant_reward_cake</x:v>
+      </x:c>
+      <x:c r="B69" s="27" t="str">
+        <x:v>Chế Bánh thưởng từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C69" s="27" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D69" s="27" t="str">
+        <x:v>food_tier_1</x:v>
+      </x:c>
+      <x:c r="E69" s="27" t="str">
+        <x:v>Thực phẩm Tier 1</x:v>
+      </x:c>
+      <x:c r="F69" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G69" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H69" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I69" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="27" t="str">
+        <x:v>bar_liquor</x:v>
+      </x:c>
+      <x:c r="B70" s="27" t="str">
+        <x:v>Chế Rượu từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C70" s="27" t="str">
+        <x:v>bar</x:v>
+      </x:c>
+      <x:c r="D70" s="27" t="str">
+        <x:v>food_tier_1</x:v>
+      </x:c>
+      <x:c r="E70" s="27" t="str">
+        <x:v>Thực phẩm Tier 1</x:v>
+      </x:c>
+      <x:c r="F70" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G70" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H70" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I70" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="27" t="str">
+        <x:v>soda_factory_monster_buff_bottle</x:v>
+      </x:c>
+      <x:c r="B71" s="27" t="str">
+        <x:v>Chế Bình nước buff từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C71" s="27" t="str">
+        <x:v>soda_factory</x:v>
+      </x:c>
+      <x:c r="D71" s="27" t="str">
+        <x:v>food_tier_1</x:v>
+      </x:c>
+      <x:c r="E71" s="27" t="str">
+        <x:v>Thực phẩm Tier 1</x:v>
+      </x:c>
+      <x:c r="F71" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G71" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H71" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I71" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="27" t="str">
+        <x:v>inn_overclock_coffee</x:v>
+      </x:c>
+      <x:c r="B72" s="27" t="str">
+        <x:v>Chế Cà phê ép xung từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C72" s="27" t="str">
+        <x:v>inn</x:v>
+      </x:c>
+      <x:c r="D72" s="27" t="str">
+        <x:v>food_tier_1</x:v>
+      </x:c>
+      <x:c r="E72" s="27" t="str">
+        <x:v>Thực phẩm Tier 1</x:v>
+      </x:c>
+      <x:c r="F72" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G72" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H72" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I72" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="27" t="str">
+        <x:v>tool_workshop_raincoat</x:v>
+      </x:c>
+      <x:c r="B73" s="27" t="str">
+        <x:v>Chế Áo mưa từ Phôi</x:v>
+      </x:c>
+      <x:c r="C73" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D73" s="27" t="str">
+        <x:v>blank_ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E73" s="27" t="str">
+        <x:v>Phôi Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F73" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G73" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H73" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I73" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="27" t="str">
+        <x:v>tool_workshop_gas_mask</x:v>
+      </x:c>
+      <x:c r="B74" s="27" t="str">
+        <x:v>Chế Mặt nạ phòng độc từ Phôi</x:v>
+      </x:c>
+      <x:c r="C74" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D74" s="27" t="str">
+        <x:v>blank_ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E74" s="27" t="str">
+        <x:v>Phôi Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F74" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G74" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H74" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I74" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="27" t="str">
+        <x:v>tool_workshop_tactics_book</x:v>
+      </x:c>
+      <x:c r="B75" s="27" t="str">
+        <x:v>Chế Sách Chiến Thuật từ Phôi</x:v>
+      </x:c>
+      <x:c r="C75" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D75" s="27" t="str">
+        <x:v>blank_ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E75" s="27" t="str">
+        <x:v>Phôi Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F75" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G75" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H75" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I75" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="27" t="str">
+        <x:v>tool_workshop_capture_ball</x:v>
+      </x:c>
+      <x:c r="B76" s="27" t="str">
+        <x:v>Chế Bóng bắt thú từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C76" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D76" s="27" t="str">
+        <x:v>blank_ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E76" s="27" t="str">
+        <x:v>Phôi Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F76" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G76" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H76" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I76" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="27" t="str">
+        <x:v>tool_workshop_capture_ball</x:v>
+      </x:c>
+      <x:c r="B77" s="27" t="str">
+        <x:v>Chế Bóng bắt thú từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C77" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D77" s="27" t="str">
+        <x:v>wood_tier_1</x:v>
+      </x:c>
+      <x:c r="E77" s="27" t="str">
+        <x:v>Gỗ Tier 1</x:v>
+      </x:c>
+      <x:c r="F77" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G77" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H77" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I77" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="27" t="str">
+        <x:v>tool_workshop_trap</x:v>
+      </x:c>
+      <x:c r="B78" s="27" t="str">
+        <x:v>Chế Bẫy từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C78" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D78" s="27" t="str">
+        <x:v>blank_ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E78" s="27" t="str">
+        <x:v>Phôi Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F78" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G78" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H78" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I78" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="27" t="str">
+        <x:v>tool_workshop_trap</x:v>
+      </x:c>
+      <x:c r="B79" s="27" t="str">
+        <x:v>Chế Bẫy từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C79" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D79" s="27" t="str">
+        <x:v>wood_tier_1</x:v>
+      </x:c>
+      <x:c r="E79" s="27" t="str">
+        <x:v>Gỗ Tier 1</x:v>
+      </x:c>
+      <x:c r="F79" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G79" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H79" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I79" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19720,6 +20510,405 @@
         <x:v>GDD 02 §1.0; docs/designs/12_Item_Catalog.md; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="27" t="str">
+        <x:v>hospital_potion</x:v>
+      </x:c>
+      <x:c r="B65" s="27" t="str">
+        <x:v>Chế Thuốc từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C65" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D65" s="27" t="str">
+        <x:v>potion</x:v>
+      </x:c>
+      <x:c r="E65" s="27" t="str">
+        <x:v>Thuốc</x:v>
+      </x:c>
+      <x:c r="F65" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G65" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H65" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I65" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="27" t="str">
+        <x:v>hospital_vaccine</x:v>
+      </x:c>
+      <x:c r="B66" s="27" t="str">
+        <x:v>Chế Vắc-xin từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C66" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D66" s="27" t="str">
+        <x:v>vaccine</x:v>
+      </x:c>
+      <x:c r="E66" s="27" t="str">
+        <x:v>Vắc-xin</x:v>
+      </x:c>
+      <x:c r="F66" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G66" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H66" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I66" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="27" t="str">
+        <x:v>hospital_tranquilizer</x:v>
+      </x:c>
+      <x:c r="B67" s="27" t="str">
+        <x:v>Chế Thuốc An Thần từ Thảo dược</x:v>
+      </x:c>
+      <x:c r="C67" s="27" t="str">
+        <x:v>hospital</x:v>
+      </x:c>
+      <x:c r="D67" s="27" t="str">
+        <x:v>tranquilizer</x:v>
+      </x:c>
+      <x:c r="E67" s="27" t="str">
+        <x:v>Thuốc An Thần</x:v>
+      </x:c>
+      <x:c r="F67" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G67" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H67" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I67" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="27" t="str">
+        <x:v>restaurant_food_drink</x:v>
+      </x:c>
+      <x:c r="B68" s="27" t="str">
+        <x:v>Chế Đồ ăn, nước uống từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C68" s="27" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D68" s="27" t="str">
+        <x:v>food_drink</x:v>
+      </x:c>
+      <x:c r="E68" s="27" t="str">
+        <x:v>Đồ ăn, nước uống</x:v>
+      </x:c>
+      <x:c r="F68" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G68" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H68" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I68" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="27" t="str">
+        <x:v>restaurant_reward_cake</x:v>
+      </x:c>
+      <x:c r="B69" s="27" t="str">
+        <x:v>Chế Bánh thưởng từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C69" s="27" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D69" s="27" t="str">
+        <x:v>reward_cake</x:v>
+      </x:c>
+      <x:c r="E69" s="27" t="str">
+        <x:v>Bánh thưởng</x:v>
+      </x:c>
+      <x:c r="F69" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G69" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H69" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I69" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="27" t="str">
+        <x:v>bar_liquor</x:v>
+      </x:c>
+      <x:c r="B70" s="27" t="str">
+        <x:v>Chế Rượu từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C70" s="27" t="str">
+        <x:v>bar</x:v>
+      </x:c>
+      <x:c r="D70" s="27" t="str">
+        <x:v>liquor</x:v>
+      </x:c>
+      <x:c r="E70" s="27" t="str">
+        <x:v>Rượu</x:v>
+      </x:c>
+      <x:c r="F70" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G70" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H70" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I70" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="27" t="str">
+        <x:v>soda_factory_monster_buff_bottle</x:v>
+      </x:c>
+      <x:c r="B71" s="27" t="str">
+        <x:v>Chế Bình nước buff từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C71" s="27" t="str">
+        <x:v>soda_factory</x:v>
+      </x:c>
+      <x:c r="D71" s="27" t="str">
+        <x:v>monster_buff_bottle</x:v>
+      </x:c>
+      <x:c r="E71" s="27" t="str">
+        <x:v>Bình nước buff</x:v>
+      </x:c>
+      <x:c r="F71" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G71" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H71" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I71" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="27" t="str">
+        <x:v>inn_overclock_coffee</x:v>
+      </x:c>
+      <x:c r="B72" s="27" t="str">
+        <x:v>Chế Cà phê ép xung từ Thực phẩm</x:v>
+      </x:c>
+      <x:c r="C72" s="27" t="str">
+        <x:v>inn</x:v>
+      </x:c>
+      <x:c r="D72" s="27" t="str">
+        <x:v>overclock_coffee</x:v>
+      </x:c>
+      <x:c r="E72" s="27" t="str">
+        <x:v>Cà phê ép xung</x:v>
+      </x:c>
+      <x:c r="F72" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G72" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H72" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I72" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="27" t="str">
+        <x:v>tool_workshop_raincoat</x:v>
+      </x:c>
+      <x:c r="B73" s="27" t="str">
+        <x:v>Chế Áo mưa từ Phôi</x:v>
+      </x:c>
+      <x:c r="C73" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D73" s="27" t="str">
+        <x:v>raincoat</x:v>
+      </x:c>
+      <x:c r="E73" s="27" t="str">
+        <x:v>Áo mưa</x:v>
+      </x:c>
+      <x:c r="F73" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G73" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H73" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I73" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="27" t="str">
+        <x:v>tool_workshop_gas_mask</x:v>
+      </x:c>
+      <x:c r="B74" s="27" t="str">
+        <x:v>Chế Mặt nạ phòng độc từ Phôi</x:v>
+      </x:c>
+      <x:c r="C74" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D74" s="27" t="str">
+        <x:v>gas_mask</x:v>
+      </x:c>
+      <x:c r="E74" s="27" t="str">
+        <x:v>Mặt nạ phòng độc</x:v>
+      </x:c>
+      <x:c r="F74" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G74" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H74" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I74" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="27" t="str">
+        <x:v>tool_workshop_tactics_book</x:v>
+      </x:c>
+      <x:c r="B75" s="27" t="str">
+        <x:v>Chế Sách Chiến Thuật từ Phôi</x:v>
+      </x:c>
+      <x:c r="C75" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D75" s="27" t="str">
+        <x:v>tactics_book</x:v>
+      </x:c>
+      <x:c r="E75" s="27" t="str">
+        <x:v>Sách Chiến Thuật</x:v>
+      </x:c>
+      <x:c r="F75" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G75" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H75" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I75" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="27" t="str">
+        <x:v>tool_workshop_capture_ball</x:v>
+      </x:c>
+      <x:c r="B76" s="27" t="str">
+        <x:v>Chế Bóng bắt thú từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C76" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D76" s="27" t="str">
+        <x:v>capture_ball</x:v>
+      </x:c>
+      <x:c r="E76" s="27" t="str">
+        <x:v>Bóng bắt thú</x:v>
+      </x:c>
+      <x:c r="F76" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G76" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H76" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I76" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="27" t="str">
+        <x:v>tool_workshop_trap</x:v>
+      </x:c>
+      <x:c r="B77" s="27" t="str">
+        <x:v>Chế Bẫy từ Phôi và Gỗ</x:v>
+      </x:c>
+      <x:c r="C77" s="27" t="str">
+        <x:v>tool_workshop</x:v>
+      </x:c>
+      <x:c r="D77" s="27" t="str">
+        <x:v>trap</x:v>
+      </x:c>
+      <x:c r="E77" s="27" t="str">
+        <x:v>Bẫy</x:v>
+      </x:c>
+      <x:c r="F77" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G77" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H77" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I77" s="27" t="str">
+        <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="27"/>
+      <x:c r="B78" s="27"/>
+      <x:c r="C78" s="27"/>
+      <x:c r="D78" s="27"/>
+      <x:c r="E78" s="27"/>
+      <x:c r="F78" s="27"/>
+      <x:c r="G78" s="27"/>
+      <x:c r="H78" s="27"/>
+      <x:c r="I78" s="27"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="27"/>
+      <x:c r="B79" s="27"/>
+      <x:c r="C79" s="27"/>
+      <x:c r="D79" s="27"/>
+      <x:c r="E79" s="27"/>
+      <x:c r="F79" s="27"/>
+      <x:c r="G79" s="27"/>
+      <x:c r="H79" s="27"/>
+      <x:c r="I79" s="27"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(sim): document supply chain scenarios
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Recddc9060dcb4af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R489745139da34290"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="R36861b422c4c41be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R0169ff10dfa94061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R7129a7dcc1724c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rdb507c7800094be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Rd73524bd9ee34af9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R15c96cea78c24fbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rdf14d986773b43e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rce618d431d9a44af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R43c4af3554df4d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R7d9c5672b50e4d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R22337f3ad2a24e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7c96130f8a8944f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rdda18c8581364a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rdcc67ddb12fa4584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Ra6626f306ce04adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rc987e85a4ba94d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="R8b6d22c4c2374484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Re5797d8d2ecc4ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="Rb7100889494441d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R7f0f6b4442374cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rf0cab4ac1a4b4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="Rf05cc1a734394fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R07b04149048d4c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R1d846f12be494d20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -103,12 +103,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -143,7 +148,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -203,6 +208,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -465,10 +476,10 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="32" t="str">
+      <x:c r="A10" s="34" t="str">
         <x:v>Sheet</x:v>
       </x:c>
-      <x:c r="B10" s="32" t="str">
+      <x:c r="B10" s="34" t="str">
         <x:v>Contents</x:v>
       </x:c>
     </x:row>
@@ -638,22 +649,22 @@
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="28" t="str">
-        <x:v>ProductionLevelMultiplier</x:v>
+        <x:v>ProductionJobDurationMultiplierByLevel</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>n.a.</x:v>
+        <x:v>1.0; 0.9; 0.8; 0.7; 0.6</x:v>
       </x:c>
       <x:c r="C7" s="28" t="str">
-        <x:v>n.a.</x:v>
+        <x:v>× thời lượng cơ sở, cấp 1–5</x:v>
       </x:c>
       <x:c r="D7" s="28" t="str">
-        <x:v>Không áp dụng</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str">
-        <x:v>Cấp Refinery đổi hiệu suất đầu ra; controller chưa áp dụng multiplier cho thời gian.</x:v>
+        <x:v>Giả định giảm 10% thời lượng mỗi cấp Producer; các giá trị cần cân bằng lại. Thời lượng sau nhân được làm tròn lên phút, tối thiểu 1 phút.</x:v>
       </x:c>
       <x:c r="F7" s="28" t="str">
-        <x:v>src/Game.Domain/Production/ProductionController.cs</x:v>
+        <x:v>src/Game.Domain/Production/ProductionController.cs; docs/superpowers/specs/2026-10-02-domain-supply-chain-design.md §HUB inventory and production</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -4061,7 +4072,7 @@
       <x:c r="G4" s="26" t="str">
         <x:v>Nguồn</x:v>
       </x:c>
-      <x:c r="H4" s="31" t="str">
+      <x:c r="H4" s="33" t="str">
         <x:v>Effect metadata</x:v>
       </x:c>
     </x:row>
@@ -5339,25 +5350,25 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="31" t="str">
+      <x:c r="A4" s="33" t="str">
         <x:v>Producer ID</x:v>
       </x:c>
-      <x:c r="B4" s="31" t="str">
+      <x:c r="B4" s="33" t="str">
         <x:v>Nhóm slot</x:v>
       </x:c>
-      <x:c r="C4" s="31" t="str">
+      <x:c r="C4" s="33" t="str">
         <x:v>Số slot</x:v>
       </x:c>
-      <x:c r="D4" s="31" t="str">
+      <x:c r="D4" s="33" t="str">
         <x:v>Đơn vị chủ</x:v>
       </x:c>
-      <x:c r="E4" s="31" t="str">
+      <x:c r="E4" s="33" t="str">
         <x:v>Sản phẩm catalog</x:v>
       </x:c>
-      <x:c r="F4" s="31" t="str">
+      <x:c r="F4" s="33" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
-      <x:c r="G4" s="31" t="str">
+      <x:c r="G4" s="33" t="str">
         <x:v>Nguồn</x:v>
       </x:c>
     </x:row>
@@ -5458,22 +5469,22 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="31" t="str">
+      <x:c r="A4" s="33" t="str">
         <x:v>Shop ID</x:v>
       </x:c>
-      <x:c r="B4" s="31" t="str">
+      <x:c r="B4" s="33" t="str">
         <x:v>Producer ID</x:v>
       </x:c>
-      <x:c r="C4" s="31" t="str">
+      <x:c r="C4" s="33" t="str">
         <x:v>Product IDs</x:v>
       </x:c>
-      <x:c r="D4" s="31" t="str">
+      <x:c r="D4" s="33" t="str">
         <x:v>Hành vi</x:v>
       </x:c>
-      <x:c r="E4" s="31" t="str">
+      <x:c r="E4" s="33" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
-      <x:c r="F4" s="31" t="str">
+      <x:c r="F4" s="33" t="str">
         <x:v>Nguồn</x:v>
       </x:c>
     </x:row>
@@ -21186,7 +21197,7 @@
         <x:v>MerchantMaximumWaitMinutes</x:v>
       </x:c>
       <x:c r="B16" s="20" t="n">
-        <x:v>180</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C16" s="20" t="str">
         <x:v>phút in-game</x:v>
@@ -21195,7 +21206,7 @@
         <x:v>Prototype</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>Bảo đảm thời gian chờ hữu hạn khi tích hợp đánh thức Trainer.</x:v>
+        <x:v>Giới hạn an toàn prototype để Trainer không chờ mãi; Merchant mới tự đánh thức Trainer khi tới.</x:v>
       </x:c>
       <x:c r="F16" s="20" t="str">
         <x:v>src/Game.Domain/Supply/Merchant.cs; GDD 02 §1.0</x:v>
@@ -21270,24 +21281,12 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
-      <x:c r="A21" s="27" t="str">
-        <x:v>MerchantSpreadLotDirection</x:v>
-      </x:c>
-      <x:c r="B21" s="27" t="str">
-        <x:v>Tăng theo lô</x:v>
-      </x:c>
-      <x:c r="C21" s="27" t="str">
-        <x:v>Quy tắc</x:v>
-      </x:c>
-      <x:c r="D21" s="27" t="str">
-        <x:v>Prototype</x:v>
-      </x:c>
-      <x:c r="E21" s="27" t="str">
-        <x:v>Spread tăng theo quy mô lô; xác nhận lại khi playtest.</x:v>
-      </x:c>
-      <x:c r="F21" s="27" t="str">
-        <x:v>src/Game.Domain/Supply/Merchant.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
-      </x:c>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs(balance): document monster simulation parameters
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,19 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7c96130f8a8944f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rdda18c8581364a1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rdcc67ddb12fa4584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Ra6626f306ce04adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rc987e85a4ba94d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="R8b6d22c4c2374484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Re5797d8d2ecc4ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="Rb7100889494441d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R7f0f6b4442374cb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rf0cab4ac1a4b4810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="Rf05cc1a734394fdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R07b04149048d4c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R1d846f12be494d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9da7bf7f12eb483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R713014c0788e4ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rdbbb5c87f6b247fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rf1443d74e06b440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R6d42e88daa924998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="R6e7a5235b1174f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Rbe78b46d03c74e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R7ad39af512ae4ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rb811455378d94e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2cc05ac78ac7415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="Rf23ef7f1d0ff4599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R2d68284f1c584a1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R96dd882fc2c44c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="Rfd6c2473828342b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="R8e7a6b7ba8e947f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R3f7735a882444285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R8859d589638b4b32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -103,12 +107,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -148,7 +157,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -214,6 +223,17 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -476,10 +496,10 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="34" t="str">
+      <x:c r="A10" s="39" t="str">
         <x:v>Sheet</x:v>
       </x:c>
-      <x:c r="B10" s="34" t="str">
+      <x:c r="B10" s="39" t="str">
         <x:v>Contents</x:v>
       </x:c>
     </x:row>
@@ -554,6 +574,18 @@
       <x:c r="B19" s="4" t="str">
         <x:v>Six shop-to-producer mappings from GDD 02/12</x:v>
       </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>Monster Catalog / Combat &amp; Capture / Zones &amp; Loot / Monster Lifecycle</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Monster, combat, capture, zone, loot and lifecycle parameters (Prototype/TBD)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4"/>
+      <x:c r="B21" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5606,6 +5638,2181 @@
       </x:c>
       <x:c r="F10" s="4" t="str">
         <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.0-1.1; docs/designs/12_Item_Catalog.md §1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="60" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Monster, Rarity, IV và cấp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Các quy tắc Monster khóa theo GDD và các hệ số runtime Prototype.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="37" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Loại dữ liệu</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Đơn vị</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="F4" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>monster.max_per_trainer</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>Số Monster mang theo</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>3 (1 Active + 2 Reserve)</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Monster/Trainer</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §2; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>monster.swap_hp_fraction</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Ngưỡng tự động Swap</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>HP fraction</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §2; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>monster.faint_behavior</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Monster 0 HP</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>Ngất, không chết; cả 3 ngất thì Trainer về HUB</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>rule</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="4" t="str">
+        <x:v>monster.level_formula</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Cấp Monster</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>20 × (Rank − 1) + ⌈Trainer Lv / 5⌉</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1; src/Game.Domain/Monsters/MonsterProgression.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>monster.iv.d</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Hệ số IV D</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="4" t="str">
+        <x:v>monster.iv.c</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>Hệ số IV C</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="4" t="str">
+        <x:v>monster.iv.b</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Hệ số IV B</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="4" t="str">
+        <x:v>monster.iv.a</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Hệ số IV A</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>monster.iv.s</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Hệ số IV S</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>monster.iv.ss</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Hệ số IV SS</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>monster.iv.sss</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Hệ số IV SSS</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>monster.rarity.common</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Hệ số Rarity Common</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters; docs/designs/04_Monster_System.md; src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>monster.rarity.rare</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Hệ số Rarity Rare</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>monster.rarity.epic</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Hệ số Rarity Epic</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>monster.rarity.legendary</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Hệ số Rarity Legendary</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>monster.rarity.ultimate</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Hệ số Rarity Ultimate</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>monster.rarity.growth_factor</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>Hệ số tăng trưởng thống kê</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStatConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4" t="str">
+        <x:v>monster.local_storage_capacity</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>Sức chứa kho Monster của Trainer</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Monster</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs MonsterStorageConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="4" t="str">
+        <x:v>monster.rarity.min_level_upgrade</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>Cấp tối thiểu tăng Rarity</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="4" t="str">
+        <x:v>monster.evolution.max_steps</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>Số lần Tiến hóa tối đa</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>steps</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="4" t="str">
+        <x:v>monster.evolution.catalog</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>Danh mục nhánh tiến hóa</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>rỗng (GDD chưa định nghĩa nhánh theo loài)</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>catalog</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/EvolutionCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="4" t="str">
+        <x:v>monster.catalog.starter</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>Loài khởi đầu</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>starter_sprout: Grass/Support, HP 300, ATK 10, DEF 10, ASPD 1, CRIT 0.05</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>definition</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="F26" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/MonsterCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="37" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B29" s="37" t="str">
+        <x:v>Bước</x:v>
+      </x:c>
+      <x:c r="C29" s="37" t="str">
+        <x:v>Tỉ lệ thành công</x:v>
+      </x:c>
+      <x:c r="D29" s="37" t="str">
+        <x:v>Đá Cường hóa</x:v>
+      </x:c>
+      <x:c r="E29" s="37" t="str">
+        <x:v>Gene Fragments</x:v>
+      </x:c>
+      <x:c r="F29" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="G29" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="4" t="str">
+        <x:v>rarity_upgrade.step_1</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>0.60</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F30" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="G30" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §4; src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="4" t="str">
+        <x:v>rarity_upgrade.step_2</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>0.40</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F31" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="G31" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §4; src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="4" t="str">
+        <x:v>rarity_upgrade.step_3</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E32" s="4" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F32" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="G32" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §4; src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="4" t="str">
+        <x:v>rarity_upgrade.step_4</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>0.10</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §4; src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="66" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Chiến đấu, Rebellion và bắt thú</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Công thức và xác suất Prototype; quy tắc hệ nguyên tố và Swap là Locked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="37" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>Đơn vị</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>combat.critical_multiplier</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>combat.max_rounds</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>rounds</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>combat.element_chart</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>9 hệ, không miễn nhiễm (0x), kháng 0.5x</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>matrix</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="4" t="str">
+        <x:v>rebellion.probability_per_missing_point</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>probability/point</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>rebellion.max_probability</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="4" t="str">
+        <x:v>rebellion.skip_weight</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>relative weight</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="4" t="str">
+        <x:v>rebellion.sleep_weight</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>relative weight</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="4" t="str">
+        <x:v>rebellion.area_aggro_weight</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>relative weight</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>rebellion.skip_actions</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>action</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>rebellion.sleep_actions</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>action</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CombatConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>capture.base_chance</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>capture.hp_depletion_bonus</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>capture.ball_tier_bonus</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>probability/tier</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>capture.trap_tier_bonus</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>probability/tier</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>capture.dexterity_scale</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>probability/point</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>capture.trapper_bonus</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>capture.rarity_penalty</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>probability/rarity</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4" t="str">
+        <x:v>capture.minimum_chance</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="4" t="str">
+        <x:v>capture.maximum_chance</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="4" t="str">
+        <x:v>capture.weak_hp_fraction</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>0.30</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>HP fraction</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="4" t="str">
+        <x:v>capture.consume_trap_on_failure</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>false (Bóng/Bẫy chỉ mất khi thành công)</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="4" t="str">
+        <x:v>capture.power_hp_weight</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>power/HP</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="4" t="str">
+        <x:v>capture.power_attack_weight</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>power/ATK</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="4" t="str">
+        <x:v>capture.power_defense_weight</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>power/DEF</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="4" t="str">
+        <x:v>capture.power_attack_speed_weight</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>power/ASPD</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="4" t="str">
+        <x:v>capture.power_critical_weight</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>power/critical</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/CaptureResolver.cs</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="60" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Zone, encounter và loot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Năm Zone khởi điểm; loot đêm/EXP đêm ×2 là Locked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="37" t="str">
+        <x:v>Zone ID</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Tên</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>Rank tối thiểu</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Phút đi bộ</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Hệ chủ đạo</x:v>
+      </x:c>
+      <x:c r="F4" s="37" t="str">
+        <x:v>Encounter/giờ</x:v>
+      </x:c>
+      <x:c r="G4" s="37" t="str">
+        <x:v>Gold/encounter</x:v>
+      </x:c>
+      <x:c r="H4" s="37" t="str">
+        <x:v>Material units/encounter</x:v>
+      </x:c>
+      <x:c r="I4" s="37" t="str">
+        <x:v>EXP/encounter</x:v>
+      </x:c>
+      <x:c r="J4" s="37" t="str">
+        <x:v>Loot đêm</x:v>
+      </x:c>
+      <x:c r="K4" s="37" t="str">
+        <x:v>EXP đêm</x:v>
+      </x:c>
+      <x:c r="L4" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="M4" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>zone_1</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>Đồng Cỏ</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>Cỏ, Nước, Đất</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I5" s="4" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="K5" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="L5" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="M5" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneCatalog.cs; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>zone_2</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>Núi Lửa</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>Lửa, Đất</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="K6" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="L6" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="M6" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneCatalog.cs; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>zone_3</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>Hầm Băng</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>Băng, Nước</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>0.667</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="K7" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="L7" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="M7" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneCatalog.cs; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="4" t="str">
+        <x:v>zone_4</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Đầm Lầy</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Độc, Nước, Cỏ</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="K8" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="L8" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="M8" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneCatalog.cs; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>zone_5</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Vực Thẳm</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Bóng tối</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="K9" s="4" t="str">
+        <x:v>×2 (Locked)</x:v>
+      </x:c>
+      <x:c r="L9" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="M9" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneCatalog.cs; docs/designs/04_Monster_System.md §2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="37" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B12" s="37" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+      <x:c r="C12" s="37" t="str">
+        <x:v>Đơn vị</x:v>
+      </x:c>
+      <x:c r="D12" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="E12" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>zone_selection.luck_gold_per_point</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>gold/point/encounter</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneSelector.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>zone_selection.expected_farm_minutes</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneSelector.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>zone_selection.capitalist_bounty_multiplier</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>src/Game.Domain/World/ZoneSelector.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>loot.luck_gold_per_point</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>gold/point</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>src/Game.Domain/World/LootResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>loot.material_pickup_chance</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>src/Game.Domain/World/LootResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>loot.backpack_capacity</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>int.MaxValue (không giới hạn trong LootConfig; sức chứa Balo ở SimConfig)</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>src/Game.Domain/World/LootResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>expedition.opponent_hp_per_experience</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>HP/EXP</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>src/Game.Domain/World/IExpeditionResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>expedition.opponent_attack</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>ATK</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>src/Game.Domain/World/IExpeditionResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>expedition.opponent_defense</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>DEF</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>src/Game.Domain/World/IExpeditionResolver.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4" t="str">
+        <x:v>expedition.opponent_attack_speed</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>ASPD</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>src/Game.Domain/World/IExpeditionResolver.cs</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="46" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Bệnh viện Thú Y, Ngân Hàng Gene, PTN, vật phẩm và chỉ số Trainer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Runtime Prototype; phí Gene Bank thu theo Payday là Khởi điểm mô phỏng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="37" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>Đơn vị</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="4" t="str">
+        <x:v>veterinary.recovery_beds</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>Monster</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.4; src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>veterinary.emergency_beds</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>Monster</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.4; src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4" t="str">
+        <x:v>veterinary.first_capture_recovery_minutes</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="4" t="str">
+        <x:v>veterinary.emergency_recovery_minutes</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>veterinary.fainted_recovery_multiplier</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="4" t="str">
+        <x:v>veterinary.emergency_price_per_ten_hp</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Gold/10 HP</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="4" t="str">
+        <x:v>veterinary.fainted_surcharge</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/VeterinaryHospital.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="4" t="str">
+        <x:v>gene_bank.capacity</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Monster</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/GeneBank.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>gene_bank.fee_per_monster_day</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Gold/Monster/day</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3; src/Game.Domain/Monsters/GeneBank.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>gene_bank.payday_days</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>days</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3; src/Game.Domain/Monsters/GeneBank.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>gene_bank.resale_price</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/GeneBank.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>genetic_lab.appraisal_price</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>genetic_lab.dismantle_gene_fragments</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>src/Game.Domain/Monsters/GeneticLab.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>item_effect.potion_heal</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>HP</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>docs/designs/12_Item_Catalog.md; src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>item_effect.buff_attack_multiplier</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>item_effect.buff_defense_multiplier</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>item_effect.buff_critical_bonus</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4" t="str">
+        <x:v>item_effect.buff_duration_minutes</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="4" t="str">
+        <x:v>item_effect.cake_rebellion_reduction</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>management points</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="4" t="str">
+        <x:v>item_effect.cake_duration_minutes</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="4" t="str">
+        <x:v>item_effect.communication_leadership_bonus</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>leadership points</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="4" t="str">
+        <x:v>item_effect.synergy_duration_minutes</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="4" t="str">
+        <x:v>item_effect.synergy_tank_defense_multiplier</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="4" t="str">
+        <x:v>item_effect.synergy_dps_critical_bonus</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="str">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="4" t="str">
+        <x:v>item_effect.synergy_support_heal</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>HP/battle</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>src/Game.Domain/Combat/MonsterItemEffects.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="4" t="str">
+        <x:v>consumable_policy.max_units_per_need</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="str">
+        <x:v>src/Game.Domain/Trainers/TrainerInventory.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="4" t="str">
+        <x:v>consumable_policy.price_sensitivity_budget_divisor</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="str">
+        <x:v>src/Game.Domain/Trainers/TrainerInventory.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="4" t="str">
+        <x:v>consumable_policy.minimum_expected_combat_risk</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>risk score</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E32" s="4" t="str">
+        <x:v>src/Game.Domain/Trainers/TrainerInventory.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="4" t="str">
+        <x:v>trainer.dexterity_range</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>8–12</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>stat</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerAttributeConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="4" t="str">
+        <x:v>trainer.luck_range</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>8–12</x:v>
+      </x:c>
+      <x:c r="C34" s="4" t="str">
+        <x:v>stat</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerAttributeConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="4" t="str">
+        <x:v>trainer.endurance_range</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>90–110</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>stat</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E35" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerAttributeConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="4" t="str">
+        <x:v>trainer.leadership_range</x:v>
+      </x:c>
+      <x:c r="B36" s="4" t="str">
+        <x:v>18–22</x:v>
+      </x:c>
+      <x:c r="C36" s="4" t="str">
+        <x:v>stat</x:v>
+      </x:c>
+      <x:c r="D36" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E36" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerAttributeConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="4" t="str">
+        <x:v>trainer.exp_base</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>EXP (cấp 1→2)</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerProgressionConfig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="4" t="str">
+        <x:v>trainer.exp_per_level</x:v>
+      </x:c>
+      <x:c r="B38" s="4" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="str">
+        <x:v>EXP/cấp</x:v>
+      </x:c>
+      <x:c r="D38" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E38" s="4" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs TrainerProgressionConfig</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(domain): complete gear itemization sub-project
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,23 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9da7bf7f12eb483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R713014c0788e4ccc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rdbbb5c87f6b247fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rf1443d74e06b440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R6d42e88daa924998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="R6e7a5235b1174f85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Rbe78b46d03c74e33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R7ad39af512ae4ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rb811455378d94e1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2cc05ac78ac7415e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="Rf23ef7f1d0ff4599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R2d68284f1c584a1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R96dd882fc2c44c0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="Rfd6c2473828342b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="R8e7a6b7ba8e947f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R3f7735a882444285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R8859d589638b4b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3715426de5d74363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R90ef52346aee491a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rf154e89348434332"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rac51b393641b444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R29e221645f1d434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rcda3ae85af904c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R98f5990eefae4a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R60e7293c93a348c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R1e027285df7941c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2e893f5939d4413c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R980726dd54d9435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R2d4666b32a304b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Rdf574639b58744a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R6c5c770457e2422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Rc2141056fb4b49a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="Rc0cb0f9d92844c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="Rea959660b7eb4624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R13555254aa5d4ccb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,8 +30,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0%"/>
+    <x:numFmt numFmtId="201" formatCode="0.####"/>
   </x:numFmts>
   <x:fonts count="13">
     <x:font>
@@ -107,7 +109,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,8 +146,33 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border>
       <x:left/>
       <x:right/>
@@ -153,11 +180,26 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="69">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -235,6 +277,73 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -584,8 +693,12 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="4"/>
-      <x:c r="B21" s="4"/>
+      <x:c r="A21" s="4" t="str">
+        <x:v>Gear &amp; Durability</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>30 gear slots, upgrade rules, durability and set/score values with GDD sources and status</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7820,6 +7933,2331 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="68" t="str">
+        <x:v>Parameter ID</x:v>
+      </x:c>
+      <x:c r="B1" s="68" t="str">
+        <x:v>Runtime Value</x:v>
+      </x:c>
+      <x:c r="C1" s="68" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D1" s="68" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E1" s="68" t="str">
+        <x:v>GDD / code source</x:v>
+      </x:c>
+      <x:c r="F1" s="68" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>gear.trainer_utility_slot_count</x:v>
+      </x:c>
+      <x:c r="B2" s="48" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>slots/Trainer</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>docs/designs/05 §1</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>Nón, Áo, Balo, Giày, Bình nước, Găng</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>gear.trainer_aura_slot_count</x:v>
+      </x:c>
+      <x:c r="B3" s="48" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>slots/Trainer</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>docs/designs/05 §1</x:v>
+      </x:c>
+      <x:c r="F3" s="47" t="str">
+        <x:v>Còi, Huy hiệu, Áo choàng, Kính, Trang Sức, Vệ tinh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>gear.monster_slot_count</x:v>
+      </x:c>
+      <x:c r="B4" s="48" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>slots/Monster</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>docs/designs/05 §1</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Vũ khí, Giáp, Vòng cổ, Lục lạc, Guốc, Lõi Nguyên tố</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>gear.team_monster_count</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Monsters/Trainer</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>docs/designs/04 §1</x:v>
+      </x:c>
+      <x:c r="F5" s="47" t="str">
+        <x:v>1 Active + 2 Reserve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>gear.total_equipment_slot_count</x:v>
+      </x:c>
+      <x:c r="B6" s="48" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>slots/Trainer + 3 Monsters</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>docs/designs/05 §1</x:v>
+      </x:c>
+      <x:c r="F6" s="47" t="str">
+        <x:v>12 Trainer + 3×6 Monster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>gear.tier_count</x:v>
+      </x:c>
+      <x:c r="B7" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>tiers</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>docs/designs/12</x:v>
+      </x:c>
+      <x:c r="F7" s="47" t="str">
+        <x:v>Tier 1–5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>gear.enhance_max_level</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>docs/designs/05 §2; 13 §4</x:v>
+      </x:c>
+      <x:c r="F8" s="47" t="str">
+        <x:v>Cường hóa +1..+20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>gear.enhance_break_from</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>target level</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>docs/designs/05 §2</x:v>
+      </x:c>
+      <x:c r="F9" s="47" t="str">
+        <x:v>Failure may break gear from +11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>gear.star_max</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>stars</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="str">
+        <x:v>docs/designs/05 §2</x:v>
+      </x:c>
+      <x:c r="F10" s="47" t="str">
+        <x:v>1–5 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
+        <x:v>gear.refine_grade_count</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>grades</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>docs/designs/05 §2</x:v>
+      </x:c>
+      <x:c r="F11" s="47" t="str">
+        <x:v>Normal→Mythic across four steps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>gear.set_threshold_2</x:v>
+      </x:c>
+      <x:c r="B12" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>equipped items</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>docs/designs/05 §3</x:v>
+      </x:c>
+      <x:c r="F12" s="47" t="str">
+        <x:v>Set bonus threshold</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>gear.set_threshold_4</x:v>
+      </x:c>
+      <x:c r="B13" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>equipped items</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>docs/designs/05 §3</x:v>
+      </x:c>
+      <x:c r="F13" s="47" t="str">
+        <x:v>Set bonus threshold</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>gear.set_threshold_6</x:v>
+      </x:c>
+      <x:c r="B14" s="48" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>equipped items</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>docs/designs/05 §3</x:v>
+      </x:c>
+      <x:c r="F14" s="47" t="str">
+        <x:v>Set bonus threshold</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>gear.aura_wear_per_action</x:v>
+      </x:c>
+      <x:c r="B15" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>points/action</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>docs/designs/05 §3</x:v>
+      </x:c>
+      <x:c r="F15" s="47" t="str">
+        <x:v>Aura gear does not wear</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>gear.broken_item_active</x:v>
+      </x:c>
+      <x:c r="B16" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>active multiplier</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>docs/designs/05 §3</x:v>
+      </x:c>
+      <x:c r="F16" s="47" t="str">
+        <x:v>Durability zero disables item</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>gear.enhance_cost_base</x:v>
+      </x:c>
+      <x:c r="B17" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>CostBase placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>gear.enhance_cost_growth</x:v>
+      </x:c>
+      <x:c r="B18" s="48" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="str">
+        <x:v>multiplier/level</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F18" s="47" t="str">
+        <x:v>CostBase×1.30^(level−1)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47" t="str">
+        <x:v>gear.enhance_break_chance</x:v>
+      </x:c>
+      <x:c r="B19" s="48" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="str">
+        <x:v>probability on failure</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F19" s="47" t="str">
+        <x:v>Does not apply when Protection Charm is used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47" t="str">
+        <x:v>gear.enhance_stone_cost</x:v>
+      </x:c>
+      <x:c r="B20" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="47" t="str">
+        <x:v>Enhancement Stone/attempt</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F20" s="47" t="str">
+        <x:v>Runtime consumes this amount on each attempt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="47" t="str">
+        <x:v>gear.enhance_protection_charm_cost</x:v>
+      </x:c>
+      <x:c r="B21" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="str">
+        <x:v>Protection Charm/attempt</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F21" s="47" t="str">
+        <x:v>Consumed only when the charm prevents a break</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="47" t="str">
+        <x:v>gear.enhance_scroll_price</x:v>
+      </x:c>
+      <x:c r="B22" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="str">
+        <x:v>Gold-equivalent</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E22" s="47" t="str">
+        <x:v>src/Game.Domain/EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F22" s="47" t="str">
+        <x:v>Legacy model field; charm price is not wired into runtime</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="47" t="str">
+        <x:v>gear.enhance_success_1</x:v>
+      </x:c>
+      <x:c r="B23" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F23" s="47" t="str">
+        <x:v>Success chance for target level +1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="47" t="str">
+        <x:v>gear.enhance_success_2</x:v>
+      </x:c>
+      <x:c r="B24" s="48" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F24" s="47" t="str">
+        <x:v>Success chance for target level +2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="47" t="str">
+        <x:v>gear.enhance_success_3</x:v>
+      </x:c>
+      <x:c r="B25" s="48" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="C25" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E25" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F25" s="47" t="str">
+        <x:v>Success chance for target level +3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="47" t="str">
+        <x:v>gear.enhance_success_4</x:v>
+      </x:c>
+      <x:c r="B26" s="48" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F26" s="47" t="str">
+        <x:v>Success chance for target level +4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="47" t="str">
+        <x:v>gear.enhance_success_5</x:v>
+      </x:c>
+      <x:c r="B27" s="48" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="C27" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D27" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E27" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F27" s="47" t="str">
+        <x:v>Success chance for target level +5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="47" t="str">
+        <x:v>gear.enhance_success_6</x:v>
+      </x:c>
+      <x:c r="B28" s="48" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="C28" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D28" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E28" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F28" s="47" t="str">
+        <x:v>Success chance for target level +6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="47" t="str">
+        <x:v>gear.enhance_success_7</x:v>
+      </x:c>
+      <x:c r="B29" s="48" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="C29" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D29" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E29" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F29" s="47" t="str">
+        <x:v>Success chance for target level +7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="47" t="str">
+        <x:v>gear.enhance_success_8</x:v>
+      </x:c>
+      <x:c r="B30" s="48" t="n">
+        <x:v>0.6499999999999999</x:v>
+      </x:c>
+      <x:c r="C30" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D30" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E30" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F30" s="47" t="str">
+        <x:v>Success chance for target level +8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="47" t="str">
+        <x:v>gear.enhance_success_9</x:v>
+      </x:c>
+      <x:c r="B31" s="48" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="C31" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D31" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E31" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F31" s="47" t="str">
+        <x:v>Success chance for target level +9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="47" t="str">
+        <x:v>gear.enhance_success_10</x:v>
+      </x:c>
+      <x:c r="B32" s="48" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="C32" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D32" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E32" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F32" s="47" t="str">
+        <x:v>Success chance for target level +10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="47" t="str">
+        <x:v>gear.enhance_success_11</x:v>
+      </x:c>
+      <x:c r="B33" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C33" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D33" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E33" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F33" s="47" t="str">
+        <x:v>Success chance for target level +11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="47" t="str">
+        <x:v>gear.enhance_success_12</x:v>
+      </x:c>
+      <x:c r="B34" s="48" t="n">
+        <x:v>0.46499999999999997</x:v>
+      </x:c>
+      <x:c r="C34" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D34" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E34" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F34" s="47" t="str">
+        <x:v>Success chance for target level +12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="47" t="str">
+        <x:v>gear.enhance_success_13</x:v>
+      </x:c>
+      <x:c r="B35" s="48" t="n">
+        <x:v>0.43</x:v>
+      </x:c>
+      <x:c r="C35" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D35" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E35" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F35" s="47" t="str">
+        <x:v>Success chance for target level +13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="47" t="str">
+        <x:v>gear.enhance_success_14</x:v>
+      </x:c>
+      <x:c r="B36" s="48" t="n">
+        <x:v>0.395</x:v>
+      </x:c>
+      <x:c r="C36" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D36" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E36" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F36" s="47" t="str">
+        <x:v>Success chance for target level +14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="47" t="str">
+        <x:v>gear.enhance_success_15</x:v>
+      </x:c>
+      <x:c r="B37" s="48" t="n">
+        <x:v>0.36</x:v>
+      </x:c>
+      <x:c r="C37" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D37" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E37" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F37" s="47" t="str">
+        <x:v>Success chance for target level +15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="47" t="str">
+        <x:v>gear.enhance_success_16</x:v>
+      </x:c>
+      <x:c r="B38" s="48" t="n">
+        <x:v>0.32499999999999996</x:v>
+      </x:c>
+      <x:c r="C38" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D38" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E38" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F38" s="47" t="str">
+        <x:v>Success chance for target level +16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="47" t="str">
+        <x:v>gear.enhance_success_17</x:v>
+      </x:c>
+      <x:c r="B39" s="48" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="C39" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D39" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E39" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F39" s="47" t="str">
+        <x:v>Success chance for target level +17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="47" t="str">
+        <x:v>gear.enhance_success_18</x:v>
+      </x:c>
+      <x:c r="B40" s="48" t="n">
+        <x:v>0.255</x:v>
+      </x:c>
+      <x:c r="C40" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D40" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E40" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F40" s="47" t="str">
+        <x:v>Success chance for target level +18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="47" t="str">
+        <x:v>gear.enhance_success_19</x:v>
+      </x:c>
+      <x:c r="B41" s="48" t="n">
+        <x:v>0.21999999999999997</x:v>
+      </x:c>
+      <x:c r="C41" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D41" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E41" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F41" s="47" t="str">
+        <x:v>Success chance for target level +19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="47" t="str">
+        <x:v>gear.enhance_success_20</x:v>
+      </x:c>
+      <x:c r="B42" s="48" t="n">
+        <x:v>0.18499999999999994</x:v>
+      </x:c>
+      <x:c r="C42" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D42" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E42" s="47" t="str">
+        <x:v>docs/designs/13 §4; EnhancementModel.cs</x:v>
+      </x:c>
+      <x:c r="F42" s="47" t="str">
+        <x:v>Success chance for target level +20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="47" t="str">
+        <x:v>gear.star_gold_base</x:v>
+      </x:c>
+      <x:c r="B43" s="48" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="C43" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D43" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E43" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F43" s="47" t="str">
+        <x:v>Star-up cost base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="47" t="str">
+        <x:v>gear.star_gold_growth</x:v>
+      </x:c>
+      <x:c r="B44" s="48" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="C44" s="47" t="str">
+        <x:v>multiplier/step</x:v>
+      </x:c>
+      <x:c r="D44" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E44" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F44" s="47" t="str">
+        <x:v>300×1.8^(step−1)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="47" t="str">
+        <x:v>gear.star_sacrifice_gold</x:v>
+      </x:c>
+      <x:c r="B45" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C45" s="47" t="str">
+        <x:v>Gold/attempt</x:v>
+      </x:c>
+      <x:c r="D45" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E45" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F45" s="47" t="str">
+        <x:v>Additional sacrifice cost</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="47" t="str">
+        <x:v>gear.star_failure_drop_from_target</x:v>
+      </x:c>
+      <x:c r="B46" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C46" s="47" t="str">
+        <x:v>target stars</x:v>
+      </x:c>
+      <x:c r="D46" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E46" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F46" s="47" t="str">
+        <x:v>Failure drops one star from target step 3 onward</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="47" t="str">
+        <x:v>gear.star_probability_step_1</x:v>
+      </x:c>
+      <x:c r="B47" s="48" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="C47" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D47" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E47" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F47" s="47" t="str">
+        <x:v>1→2 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="47" t="str">
+        <x:v>gear.star_probability_step_2</x:v>
+      </x:c>
+      <x:c r="B48" s="48" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="C48" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D48" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E48" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F48" s="47" t="str">
+        <x:v>2→3 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="47" t="str">
+        <x:v>gear.star_probability_step_3</x:v>
+      </x:c>
+      <x:c r="B49" s="48" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="C49" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D49" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E49" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F49" s="47" t="str">
+        <x:v>3→4 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="47" t="str">
+        <x:v>gear.star_probability_step_4</x:v>
+      </x:c>
+      <x:c r="B50" s="48" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="C50" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D50" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E50" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F50" s="47" t="str">
+        <x:v>4→5 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="47" t="str">
+        <x:v>gear.star_probability_step_5_unreachable</x:v>
+      </x:c>
+      <x:c r="B51" s="48" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="C51" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D51" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E51" s="47" t="str">
+        <x:v>docs/designs/13 §4 versus 05 §2</x:v>
+      </x:c>
+      <x:c r="F51" s="47" t="str">
+        <x:v>GDD 13 gives a fifth probability; GDD 05 caps at 5 stars</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="47" t="str">
+        <x:v>gear.refine_gold_base</x:v>
+      </x:c>
+      <x:c r="B52" s="48" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C52" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D52" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E52" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F52" s="47" t="str">
+        <x:v>First refine attempt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="47" t="str">
+        <x:v>gear.refine_gold_growth</x:v>
+      </x:c>
+      <x:c r="B53" s="48" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="C53" s="47" t="str">
+        <x:v>multiplier/step</x:v>
+      </x:c>
+      <x:c r="D53" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E53" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F53" s="47" t="str">
+        <x:v>1000×2.5^(step−1)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="47" t="str">
+        <x:v>gear.refine_probability_step_1</x:v>
+      </x:c>
+      <x:c r="B54" s="48" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="C54" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D54" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E54" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F54" s="47" t="str">
+        <x:v>Normal→Refined</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="47" t="str">
+        <x:v>gear.refine_probability_step_2</x:v>
+      </x:c>
+      <x:c r="B55" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C55" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D55" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E55" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F55" s="47" t="str">
+        <x:v>Refined→Rare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="47" t="str">
+        <x:v>gear.refine_probability_step_3</x:v>
+      </x:c>
+      <x:c r="B56" s="48" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C56" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D56" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E56" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F56" s="47" t="str">
+        <x:v>Rare→Epic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="47" t="str">
+        <x:v>gear.refine_probability_step_4</x:v>
+      </x:c>
+      <x:c r="B57" s="48" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="C57" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D57" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E57" s="47" t="str">
+        <x:v>docs/designs/13 §4; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F57" s="47" t="str">
+        <x:v>Epic→Mythic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="47" t="str">
+        <x:v>gear.refine_crystal_cost</x:v>
+      </x:c>
+      <x:c r="B58" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C58" s="47" t="str">
+        <x:v>World Boss Crystal/attempt</x:v>
+      </x:c>
+      <x:c r="D58" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E58" s="47" t="str">
+        <x:v>docs/designs/05 §2; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F58" s="47" t="str">
+        <x:v>Quantity unspecified in GDD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="47" t="str">
+        <x:v>gear.refine_water_cost</x:v>
+      </x:c>
+      <x:c r="B59" s="48" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C59" s="47" t="str">
+        <x:v>Distilled Water/attempt</x:v>
+      </x:c>
+      <x:c r="D59" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E59" s="47" t="str">
+        <x:v>docs/designs/05 §2; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F59" s="47" t="str">
+        <x:v>Quantity unspecified; distilled water is 10× price</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="47" t="str">
+        <x:v>gear.enhance_per_level_fraction</x:v>
+      </x:c>
+      <x:c r="B60" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C60" s="47" t="str">
+        <x:v>Tier 1 base stat/level</x:v>
+      </x:c>
+      <x:c r="D60" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E60" s="47" t="str">
+        <x:v>docs/designs/05 §2; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F60" s="47" t="str">
+        <x:v>Flat addition before star/refine multipliers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="47" t="str">
+        <x:v>gear.star_fraction_per_star</x:v>
+      </x:c>
+      <x:c r="B61" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C61" s="47" t="str">
+        <x:v>fraction/star</x:v>
+      </x:c>
+      <x:c r="D61" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E61" s="47" t="str">
+        <x:v>docs/designs/05 §2; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F61" s="47" t="str">
+        <x:v>Magnitude unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="47" t="str">
+        <x:v>gear.unit_stat_attack</x:v>
+      </x:c>
+      <x:c r="B62" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C62" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D62" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E62" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F62" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="47" t="str">
+        <x:v>gear.unit_stat_defense</x:v>
+      </x:c>
+      <x:c r="B63" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C63" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D63" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E63" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F63" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="47" t="str">
+        <x:v>gear.unit_stat_hp</x:v>
+      </x:c>
+      <x:c r="B64" s="48" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C64" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D64" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E64" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F64" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="47" t="str">
+        <x:v>gear.unit_stat_attack_speed</x:v>
+      </x:c>
+      <x:c r="B65" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C65" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D65" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E65" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F65" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="47" t="str">
+        <x:v>gear.unit_stat_critical_chance</x:v>
+      </x:c>
+      <x:c r="B66" s="48" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C66" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D66" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E66" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F66" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="47" t="str">
+        <x:v>gear.unit_stat_backpack_capacity</x:v>
+      </x:c>
+      <x:c r="B67" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C67" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D67" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E67" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F67" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="47" t="str">
+        <x:v>gear.unit_stat_night_vision</x:v>
+      </x:c>
+      <x:c r="B68" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C68" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D68" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E68" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F68" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="47" t="str">
+        <x:v>gear.unit_stat_hydration_decay_reduction</x:v>
+      </x:c>
+      <x:c r="B69" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C69" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D69" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E69" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F69" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="47" t="str">
+        <x:v>gear.unit_stat_mining_speed</x:v>
+      </x:c>
+      <x:c r="B70" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C70" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D70" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E70" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F70" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="47" t="str">
+        <x:v>gear.unit_stat_aura_attack_multiplier</x:v>
+      </x:c>
+      <x:c r="B71" s="48" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C71" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D71" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E71" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F71" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="47" t="str">
+        <x:v>gear.unit_stat_aura_defense_multiplier</x:v>
+      </x:c>
+      <x:c r="B72" s="48" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C72" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D72" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E72" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F72" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="47" t="str">
+        <x:v>gear.unit_stat_aura_crit_chance</x:v>
+      </x:c>
+      <x:c r="B73" s="48" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C73" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D73" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E73" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F73" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="47" t="str">
+        <x:v>gear.unit_stat_stamina_decay_reduction</x:v>
+      </x:c>
+      <x:c r="B74" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C74" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D74" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E74" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F74" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="47" t="str">
+        <x:v>gear.unit_stat_move_speed_multiplier</x:v>
+      </x:c>
+      <x:c r="B75" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C75" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D75" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E75" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F75" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="47" t="str">
+        <x:v>gear.unit_stat_weather_resist</x:v>
+      </x:c>
+      <x:c r="B76" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C76" s="47" t="str">
+        <x:v>stat/Tier 1</x:v>
+      </x:c>
+      <x:c r="D76" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E76" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F76" s="47" t="str">
+        <x:v>Base stat placeholder; per-level use scales from Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="47" t="str">
+        <x:v>gear.refine_multiplier_0</x:v>
+      </x:c>
+      <x:c r="B77" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C77" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D77" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E77" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F77" s="47" t="str">
+        <x:v>Effective stat multiplier at refine grade 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="47" t="str">
+        <x:v>gear.refine_multiplier_1</x:v>
+      </x:c>
+      <x:c r="B78" s="48" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="C78" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D78" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E78" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F78" s="47" t="str">
+        <x:v>Effective stat multiplier at refine grade 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="47" t="str">
+        <x:v>gear.refine_multiplier_2</x:v>
+      </x:c>
+      <x:c r="B79" s="48" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="C79" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D79" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E79" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F79" s="47" t="str">
+        <x:v>Effective stat multiplier at refine grade 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="47" t="str">
+        <x:v>gear.refine_multiplier_3</x:v>
+      </x:c>
+      <x:c r="B80" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C80" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D80" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E80" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F80" s="47" t="str">
+        <x:v>Effective stat multiplier at refine grade 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="47" t="str">
+        <x:v>gear.refine_multiplier_4</x:v>
+      </x:c>
+      <x:c r="B81" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C81" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D81" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E81" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F81" s="47" t="str">
+        <x:v>Effective stat multiplier at refine grade 4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="47" t="str">
+        <x:v>gear.monster_max_durability</x:v>
+      </x:c>
+      <x:c r="B82" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C82" s="47" t="str">
+        <x:v>points</x:v>
+      </x:c>
+      <x:c r="D82" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E82" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F82" s="47" t="str">
+        <x:v>GDD does not specify capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="47" t="str">
+        <x:v>gear.utility_max_durability</x:v>
+      </x:c>
+      <x:c r="B83" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C83" s="47" t="str">
+        <x:v>points</x:v>
+      </x:c>
+      <x:c r="D83" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E83" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F83" s="47" t="str">
+        <x:v>GDD does not specify capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="47" t="str">
+        <x:v>gear.aura_max_durability</x:v>
+      </x:c>
+      <x:c r="B84" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C84" s="47" t="str">
+        <x:v>points</x:v>
+      </x:c>
+      <x:c r="D84" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E84" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F84" s="47" t="str">
+        <x:v>Storage placeholder; Aura never wears</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="47" t="str">
+        <x:v>gear.monster_wear_per_action</x:v>
+      </x:c>
+      <x:c r="B85" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C85" s="47" t="str">
+        <x:v>points/action</x:v>
+      </x:c>
+      <x:c r="D85" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E85" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F85" s="47" t="str">
+        <x:v>Amount unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="47" t="str">
+        <x:v>gear.monster_wear_per_hit</x:v>
+      </x:c>
+      <x:c r="B86" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C86" s="47" t="str">
+        <x:v>points/hit</x:v>
+      </x:c>
+      <x:c r="D86" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E86" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F86" s="47" t="str">
+        <x:v>Amount unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="47" t="str">
+        <x:v>gear.utility_wear_per_farm_hour</x:v>
+      </x:c>
+      <x:c r="B87" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C87" s="47" t="str">
+        <x:v>points/hour</x:v>
+      </x:c>
+      <x:c r="D87" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E87" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F87" s="47" t="str">
+        <x:v>Weather currently factor 1 until sub-project 6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="47" t="str">
+        <x:v>gear.utility_weather_factor_default</x:v>
+      </x:c>
+      <x:c r="B88" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C88" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D88" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E88" s="47" t="str">
+        <x:v>src/Game.Domain/Hub/HubWorld.Gear.cs</x:v>
+      </x:c>
+      <x:c r="F88" s="47" t="str">
+        <x:v>Weather integration is owned by sub-project 6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="47" t="str">
+        <x:v>gear.repair_gold_per_durability</x:v>
+      </x:c>
+      <x:c r="B89" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C89" s="47" t="str">
+        <x:v>Gold/point</x:v>
+      </x:c>
+      <x:c r="D89" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E89" s="47" t="str">
+        <x:v>docs/designs/05 §3; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F89" s="47" t="str">
+        <x:v>Repair sink placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="47" t="str">
+        <x:v>gear.night_vision_minimum_tier</x:v>
+      </x:c>
+      <x:c r="B90" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C90" s="47" t="str">
+        <x:v>tier</x:v>
+      </x:c>
+      <x:c r="D90" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E90" s="47" t="str">
+        <x:v>docs/designs/05 §1; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F90" s="47" t="str">
+        <x:v>GDD says from one tier; exact tier unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="47" t="str">
+        <x:v>gear.acceptance_gold_fraction</x:v>
+      </x:c>
+      <x:c r="B91" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C91" s="47" t="str">
+        <x:v>fraction of cash</x:v>
+      </x:c>
+      <x:c r="D91" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E91" s="47" t="str">
+        <x:v>docs/designs/05 §1; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F91" s="47" t="str">
+        <x:v>Price acceptance threshold</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="47" t="str">
+        <x:v>gear.buyback_fraction</x:v>
+      </x:c>
+      <x:c r="B92" s="48" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="C92" s="47" t="str">
+        <x:v>fraction of offer price</x:v>
+      </x:c>
+      <x:c r="D92" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E92" s="47" t="str">
+        <x:v>docs/designs/05 §1; GearConfig.cs</x:v>
+      </x:c>
+      <x:c r="F92" s="47" t="str">
+        <x:v>Buyback price placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="47" t="str">
+        <x:v>gear.score_weight_hp</x:v>
+      </x:c>
+      <x:c r="B93" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C93" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D93" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E93" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F93" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="47" t="str">
+        <x:v>gear.score_weight_attack_speed</x:v>
+      </x:c>
+      <x:c r="B94" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C94" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D94" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E94" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F94" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="47" t="str">
+        <x:v>gear.score_weight_critical_chance</x:v>
+      </x:c>
+      <x:c r="B95" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C95" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D95" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E95" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F95" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="47" t="str">
+        <x:v>gear.score_weight_hydration_decay_reduction</x:v>
+      </x:c>
+      <x:c r="B96" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C96" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D96" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E96" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F96" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="47" t="str">
+        <x:v>gear.score_weight_mining_speed</x:v>
+      </x:c>
+      <x:c r="B97" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C97" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D97" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E97" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F97" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="47" t="str">
+        <x:v>gear.score_weight_aura_attack_multiplier</x:v>
+      </x:c>
+      <x:c r="B98" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C98" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D98" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E98" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F98" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="47" t="str">
+        <x:v>gear.score_weight_aura_defense_multiplier</x:v>
+      </x:c>
+      <x:c r="B99" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C99" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D99" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E99" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F99" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="47" t="str">
+        <x:v>gear.score_weight_aura_crit_chance</x:v>
+      </x:c>
+      <x:c r="B100" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C100" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D100" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E100" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F100" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="47" t="str">
+        <x:v>gear.score_weight_stamina_decay_reduction</x:v>
+      </x:c>
+      <x:c r="B101" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C101" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D101" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E101" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F101" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="47" t="str">
+        <x:v>gear.score_weight_move_speed_multiplier</x:v>
+      </x:c>
+      <x:c r="B102" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C102" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D102" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E102" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F102" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="47" t="str">
+        <x:v>gear.score_weight_weather_resist</x:v>
+      </x:c>
+      <x:c r="B103" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C103" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D103" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E103" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F103" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="47" t="str">
+        <x:v>gear.score_weight_night_vision</x:v>
+      </x:c>
+      <x:c r="B104" s="48" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C104" s="47" t="str">
+        <x:v>score per stat unit</x:v>
+      </x:c>
+      <x:c r="D104" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E104" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F104" s="47" t="str">
+        <x:v>Gear Score conversion placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="47" t="str">
+        <x:v>gear.score_weight_attack</x:v>
+      </x:c>
+      <x:c r="B105" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C105" s="47" t="str">
+        <x:v>score/stat</x:v>
+      </x:c>
+      <x:c r="D105" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E105" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F105" s="47" t="str">
+        <x:v>Direct score sum</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="47" t="str">
+        <x:v>gear.score_weight_defense</x:v>
+      </x:c>
+      <x:c r="B106" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C106" s="47" t="str">
+        <x:v>score/stat</x:v>
+      </x:c>
+      <x:c r="D106" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E106" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F106" s="47" t="str">
+        <x:v>Direct score sum</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="47" t="str">
+        <x:v>gear.score_weight_backpack_capacity</x:v>
+      </x:c>
+      <x:c r="B107" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C107" s="47" t="str">
+        <x:v>score/unit</x:v>
+      </x:c>
+      <x:c r="D107" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E107" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearScore.cs</x:v>
+      </x:c>
+      <x:c r="F107" s="47" t="str">
+        <x:v>Direct score sum</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="47" t="str">
+        <x:v>gear.monster_set_alpha_2_attack</x:v>
+      </x:c>
+      <x:c r="B108" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C108" s="47" t="str">
+        <x:v>Attack</x:v>
+      </x:c>
+      <x:c r="D108" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E108" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F108" s="47" t="str">
+        <x:v>2-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="47" t="str">
+        <x:v>gear.monster_set_alpha_4_defense</x:v>
+      </x:c>
+      <x:c r="B109" s="48" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C109" s="47" t="str">
+        <x:v>Defense</x:v>
+      </x:c>
+      <x:c r="D109" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E109" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F109" s="47" t="str">
+        <x:v>4-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="47" t="str">
+        <x:v>gear.monster_set_alpha_4_hp</x:v>
+      </x:c>
+      <x:c r="B110" s="48" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C110" s="47" t="str">
+        <x:v>HP</x:v>
+      </x:c>
+      <x:c r="D110" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E110" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F110" s="47" t="str">
+        <x:v>4-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="47" t="str">
+        <x:v>gear.monster_set_alpha_6_attack</x:v>
+      </x:c>
+      <x:c r="B111" s="48" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C111" s="47" t="str">
+        <x:v>Attack</x:v>
+      </x:c>
+      <x:c r="D111" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E111" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F111" s="47" t="str">
+        <x:v>6-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="47" t="str">
+        <x:v>gear.monster_set_alpha_6_critical_chance</x:v>
+      </x:c>
+      <x:c r="B112" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C112" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D112" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E112" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F112" s="47" t="str">
+        <x:v>6-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="47" t="str">
+        <x:v>gear.aura_set_alpha_2_attack_multiplier</x:v>
+      </x:c>
+      <x:c r="B113" s="48" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="C113" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D113" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E113" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F113" s="47" t="str">
+        <x:v>2-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="47" t="str">
+        <x:v>gear.aura_set_alpha_4_defense_multiplier</x:v>
+      </x:c>
+      <x:c r="B114" s="48" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="C114" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D114" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E114" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F114" s="47" t="str">
+        <x:v>4-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="47" t="str">
+        <x:v>gear.aura_set_alpha_6_crit</x:v>
+      </x:c>
+      <x:c r="B115" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C115" s="47" t="str">
+        <x:v>probability</x:v>
+      </x:c>
+      <x:c r="D115" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E115" s="47" t="str">
+        <x:v>src/Game.Domain/Gear/GearCatalog.cs</x:v>
+      </x:c>
+      <x:c r="F115" s="47" t="str">
+        <x:v>6-piece set bonus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116"/>
+      <x:c r="B116"/>
+      <x:c r="C116"/>
+      <x:c r="D116"/>
+      <x:c r="E116"/>
+      <x:c r="F116"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
feat(domain): complete finance sub-project
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,24 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3715426de5d74363"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R90ef52346aee491a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rf154e89348434332"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rac51b393641b444d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R29e221645f1d434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rcda3ae85af904c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R98f5990eefae4a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R60e7293c93a348c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R1e027285df7941c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2e893f5939d4413c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R980726dd54d9435b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R2d4666b32a304b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Rdf574639b58744a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R6c5c770457e2422a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Rc2141056fb4b49a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="Rc0cb0f9d92844c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="Rea959660b7eb4624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R13555254aa5d4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R716e073dfa344d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R13ca191ce3be4d86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rc42b3a857a0a4e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R3c3936f02bd34218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rfdfb14de4f064dc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rfd3553c4591f4861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R68a0620aca1a4ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="Rfb692cb95af746ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R5244ca087e0543b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2bf02e6416754df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R6ffa66d550de48f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="Re9185e1838ec4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R5fcdb35ce74f4e64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R8cc50aad0f57484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Re5c6d402e4744ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R7b296563f2584f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="Rc78c37a44f46440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R90293174c2b5447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="R42d6f250a77442a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -109,12 +110,32 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -199,7 +220,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="89">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -343,6 +364,50 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -700,6 +765,14 @@
         <x:v>30 gear slots, upgrade rules, durability and set/score values with GDD sources and status</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Trainer loans, reverse loans, stock market and Gene Bank fees with GDD source and status</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7946,22 +8019,22 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="68" t="str">
+      <x:c r="A1" s="88" t="str">
         <x:v>Parameter ID</x:v>
       </x:c>
-      <x:c r="B1" s="68" t="str">
+      <x:c r="B1" s="88" t="str">
         <x:v>Runtime Value</x:v>
       </x:c>
-      <x:c r="C1" s="68" t="str">
+      <x:c r="C1" s="88" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="D1" s="68" t="str">
+      <x:c r="D1" s="88" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="E1" s="68" t="str">
+      <x:c r="E1" s="88" t="str">
         <x:v>GDD / code source</x:v>
       </x:c>
-      <x:c r="F1" s="68" t="str">
+      <x:c r="F1" s="88" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -10252,6 +10325,583 @@
       <x:c r="D116"/>
       <x:c r="E116"/>
       <x:c r="F116"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="88" t="str">
+        <x:v>Parameter ID</x:v>
+      </x:c>
+      <x:c r="B1" s="88" t="str">
+        <x:v>Runtime Value</x:v>
+      </x:c>
+      <x:c r="C1" s="88" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D1" s="88" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E1" s="88" t="str">
+        <x:v>GDD / code source</x:v>
+      </x:c>
+      <x:c r="F1" s="88" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>loan.interest_per_payday</x:v>
+      </x:c>
+      <x:c r="B2" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>fraction/Payday</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §12: default 10%; adjustable 5-40%</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>Adjustable range 5–40%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>loan.monthly_wage_limit_multiplier</x:v>
+      </x:c>
+      <x:c r="B3" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>monthly wages</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §12: default credit limit 2 monthly wages</x:v>
+      </x:c>
+      <x:c r="F3" s="47" t="str">
+        <x:v>HUB credit limit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>loan.income_repayment_fraction</x:v>
+      </x:c>
+      <x:c r="B4" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>fraction</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §12: apply 50% of income and wages to debt</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Share of eligible Trainer income applied to debt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>loan.over_limit_paydays_to_strike</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Paydays</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §12: strike after exceeding limit for two consecutive Paydays</x:v>
+      </x:c>
+      <x:c r="F5" s="47" t="str">
+        <x:v>Consecutive Paydays beyond limit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>reverse_loan.cash_limit_fraction</x:v>
+      </x:c>
+      <x:c r="B6" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>fraction of lender cash</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2; docs/designs/13_Balance_Parameters.md §13: about 50% of each Rank V Trainer's cash</x:v>
+      </x:c>
+      <x:c r="F6" s="47" t="str">
+        <x:v>Rank V Trainer lenders</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>reverse_loan.interest_per_payday</x:v>
+      </x:c>
+      <x:c r="B7" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>fraction/Payday</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2; docs/designs/13_Balance_Parameters.md §13: 5% per Payday</x:v>
+      </x:c>
+      <x:c r="F7" s="47" t="str">
+        <x:v>Interest owed to Trainer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>reverse_loan.term_paydays</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Paydays</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2; docs/designs/13_Balance_Parameters.md §13: due in 1-2 Paydays</x:v>
+      </x:c>
+      <x:c r="F8" s="47" t="str">
+        <x:v>Within GDD 1–2 Payday term</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>stock.daily_volatility</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>fraction/day</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: random ±3%/day; docs/designs/13_Balance_Parameters.md §3</x:v>
+      </x:c>
+      <x:c r="F9" s="47" t="str">
+        <x:v>Seeded random noise ±3%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>stock.traffic_sensitivity</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>fraction per traffic fraction</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: 0.5 × Traffic change</x:v>
+      </x:c>
+      <x:c r="F10" s="47" t="str">
+        <x:v>GDD coefficient</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
+        <x:v>stock.order_impact_coefficient</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>fraction per net shares/outstanding</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: coefficient k is unspecified; Prototype value</x:v>
+      </x:c>
+      <x:c r="F11" s="47" t="str">
+        <x:v>GDD coefficient k unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>stock.dividend_rate</x:v>
+      </x:c>
+      <x:c r="B12" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>fraction of 15-day revenue</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3: 10% every 15 days</x:v>
+      </x:c>
+      <x:c r="F12" s="47" t="str">
+        <x:v>Dividend pool every 15 days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>stock.dividend_period_days</x:v>
+      </x:c>
+      <x:c r="B13" s="48" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>days</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3: every 15 days</x:v>
+      </x:c>
+      <x:c r="F13" s="47" t="str">
+        <x:v>Dividend window</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>stock.target_annual_yield</x:v>
+      </x:c>
+      <x:c r="B14" s="48" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>fraction/year</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3: IPO target yield 8%/year</x:v>
+      </x:c>
+      <x:c r="F14" s="47" t="str">
+        <x:v>IPO share count yield target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>stock.realized_profit_tax_rate</x:v>
+      </x:c>
+      <x:c r="B15" s="48" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>fraction of realized gains</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §3: 30%; losses are untaxed</x:v>
+      </x:c>
+      <x:c r="F15" s="47" t="str">
+        <x:v>Losses are untaxed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>stock.transaction_fee_rate</x:v>
+      </x:c>
+      <x:c r="B16" s="48" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>fraction of trade value</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3 says each Trainer transaction pays an exchange fee; rate TBD, Prototype value</x:v>
+      </x:c>
+      <x:c r="F16" s="47" t="str">
+        <x:v>Rate is unspecified by GDD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>stock.opening_share_price</x:v>
+      </x:c>
+      <x:c r="B17" s="48" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Gold/share</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>Prototype base quote for initial IPO pricing</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>Initial IPO quote</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>stock.hub_locked_share_fraction</x:v>
+      </x:c>
+      <x:c r="B18" s="48" t="n">
+        <x:v>0.51</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="str">
+        <x:v>fraction of issued shares</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3 and docs/designs/13_Balance_Parameters.md §3: HUB holds locked 51%</x:v>
+      </x:c>
+      <x:c r="F18" s="47" t="str">
+        <x:v>HUB holds 51% locked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47" t="str">
+        <x:v>stock.minimum_ipo_facility_level</x:v>
+      </x:c>
+      <x:c r="B19" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="str">
+        <x:v>facility levels</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3 requires an eligible building level; threshold not specified, Prototype</x:v>
+      </x:c>
+      <x:c r="F19" s="47" t="str">
+        <x:v>GDD threshold unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47" t="str">
+        <x:v>stock.listings_per_exchange_level</x:v>
+      </x:c>
+      <x:c r="B20" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="47" t="str">
+        <x:v>listings/Exchange level</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: Exchange level controls listings; rate not specified, Prototype</x:v>
+      </x:c>
+      <x:c r="F20" s="47" t="str">
+        <x:v>GDD scaling unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="47" t="str">
+        <x:v>stock.ai_common_buy_fraction</x:v>
+      </x:c>
+      <x:c r="B21" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="str">
+        <x:v>available float fraction/day</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: Common tends to go all-in/borrow; exact fraction is Prototype</x:v>
+      </x:c>
+      <x:c r="F21" s="47" t="str">
+        <x:v>Common tends to go all-in or borrow; exact fraction unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="47" t="str">
+        <x:v>stock.ai_ultimate_buy_fraction</x:v>
+      </x:c>
+      <x:c r="B22" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="str">
+        <x:v>available float fraction/day</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E22" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: Ultimate prefers blue-chip; exact fraction is Prototype</x:v>
+      </x:c>
+      <x:c r="F22" s="47" t="str">
+        <x:v>Ultimate prefers blue-chip shares; exact fraction unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="47" t="str">
+        <x:v>stock.ai_capitalist_trade_fraction</x:v>
+      </x:c>
+      <x:c r="B23" s="48" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="str">
+        <x:v>held shares fraction/day</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: Capitalist day-trades; exact fraction is Prototype</x:v>
+      </x:c>
+      <x:c r="F23" s="47" t="str">
+        <x:v>Capitalist day-trades; exact fraction unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="47" t="str">
+        <x:v>stock.ai_timid_panic_drop_3day</x:v>
+      </x:c>
+      <x:c r="B24" s="48" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>fraction decline/3 days</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §3: Timid panic-sells; threshold Prototype</x:v>
+      </x:c>
+      <x:c r="F24" s="47" t="str">
+        <x:v>Timid panic-sell threshold unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="47" t="str">
+        <x:v>gene_bank.capacity</x:v>
+      </x:c>
+      <x:c r="B25" s="48" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C25" s="47" t="str">
+        <x:v>Monsters</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E25" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §13 and docs/designs/02_HUB_Economy_Infrastructure.md §2; capacity/resale price are prototype settings.</x:v>
+      </x:c>
+      <x:c r="F25" s="47" t="str">
+        <x:v>GDD capacity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="47" t="str">
+        <x:v>gene_bank.fee_per_monster_day</x:v>
+      </x:c>
+      <x:c r="B26" s="48" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>Gold/Monster/day</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §13 and docs/designs/02_HUB_Economy_Infrastructure.md §2; capacity/resale price are prototype settings.</x:v>
+      </x:c>
+      <x:c r="F26" s="47" t="str">
+        <x:v>Assessed for 30-day Payday cycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="47" t="str">
+        <x:v>gene_bank.payday_days</x:v>
+      </x:c>
+      <x:c r="B27" s="48" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C27" s="47" t="str">
+        <x:v>days</x:v>
+      </x:c>
+      <x:c r="D27" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E27" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §13 and docs/designs/02_HUB_Economy_Infrastructure.md §2; capacity/resale price are prototype settings.</x:v>
+      </x:c>
+      <x:c r="F27" s="47" t="str">
+        <x:v>Fee assessment period</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="47" t="str">
+        <x:v>gene_bank.resale_price</x:v>
+      </x:c>
+      <x:c r="B28" s="48" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C28" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D28" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E28" s="47" t="str">
+        <x:v>docs/designs/13_Balance_Parameters.md §13 and docs/designs/02_HUB_Economy_Infrastructure.md §2; capacity/resale price are prototype settings.</x:v>
+      </x:c>
+      <x:c r="F28" s="47" t="str">
+        <x:v>Prototype setting; not used for fee settlement</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(domain): complete progression and events sub-project
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,25 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R716e073dfa344d7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R13ca191ce3be4d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rc42b3a857a0a4e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R3c3936f02bd34218"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rfdfb14de4f064dc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rfd3553c4591f4861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R68a0620aca1a4ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="Rfb692cb95af746ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R5244ca087e0543b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R2bf02e6416754df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R6ffa66d550de48f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="Re9185e1838ec4af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R5fcdb35ce74f4e64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R8cc50aad0f57484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Re5c6d402e4744ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R7b296563f2584f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="Rc78c37a44f46440c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R90293174c2b5447a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="R42d6f250a77442a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R10789b43e96948e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R59a974accfaf4b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Re260193becfc463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R7fd798922ae34acc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rbbc0f1b7b1dd4a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rf86d881f8a6e44ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R6a7f9ba2aaed4612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R7885bf1965554c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rd582fe2f35e948b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rdefc22f573124f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R428c4efb8bed4ec7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R133cc75eee1f412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Refd1053fecba4a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R7a9814b8647b4fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Rd07e849ca9c44737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R13684d74a9b34650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R4cd1090cdf6743d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R2245c98daa2d4789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="Rb9995bbfcb994fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP6 Progression &amp; Events" sheetId="20" r:id="Rb98afae9c0854aa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,11 +32,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="0.####"/>
+    <x:numFmt numFmtId="202" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -109,13 +111,74 @@
       <x:color rgb="FF1F1F1F"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -220,7 +283,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="174">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -410,11 +473,241 @@
     <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -773,6 +1066,14 @@
         <x:v>Trainer loans, reverse loans, stock market and Gene Bank fees with GDD source and status</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>SP6 Progression &amp; Events</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>See SP6 Progression &amp; Events sheet; all parameters carry status and source.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5537,6 +5838,108 @@
       </x:c>
       <x:c r="F60" t="str">
         <x:v>src/Game.Domain/Production/ProductionController.cs; docs/designs/02_HUB_Economy_Infrastructure.md §1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>wood_ingot</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Phôi Gỗ</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>Gold/đơn vị</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>Construction material; Prototype mapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>stone_ingot</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>Phôi Đá</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>Gold/đơn vị</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>Prototype maps Ore Tier 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>iron_ingot</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>Phôi Sắt</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>Gold/đơn vị</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>Prototype maps Ore Tier 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>boss_core</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>Lõi Boss</x:v>
+      </x:c>
+      <x:c r="C64"/>
+      <x:c r="D64" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>Gold/đơn vị</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>Siege victory loot; Prototype quantity in event config</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12431,6 +12834,3043 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="85" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="169" t="str">
+        <x:v>SP6 · Progression, Reputation &amp; Events</x:v>
+      </x:c>
+      <x:c r="B1" s="169"/>
+      <x:c r="C1" s="169"/>
+      <x:c r="D1" s="169"/>
+      <x:c r="E1" s="169"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="173" t="str">
+        <x:v>Stable ID</x:v>
+      </x:c>
+      <x:c r="B2" s="173" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C2" s="173" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D2" s="173" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E2" s="173" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>progression.zone_1.population_cap</x:v>
+      </x:c>
+      <x:c r="B3" s="98" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>Trainers</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>progression.zone_1.rank_count_gate</x:v>
+      </x:c>
+      <x:c r="B4" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Trainers at Rank &gt;= Zone</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>progression.zone_2.population_cap</x:v>
+      </x:c>
+      <x:c r="B5" s="98" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Trainers</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>progression.zone_2.rank_count_gate</x:v>
+      </x:c>
+      <x:c r="B6" s="98" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>Trainers at Rank &gt;= Zone</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>progression.zone_3.population_cap</x:v>
+      </x:c>
+      <x:c r="B7" s="98" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>Trainers</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>progression.zone_3.rank_count_gate</x:v>
+      </x:c>
+      <x:c r="B8" s="98" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Trainers at Rank &gt;= Zone</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>progression.zone_4.population_cap</x:v>
+      </x:c>
+      <x:c r="B9" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>Trainers</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>progression.zone_4.rank_count_gate</x:v>
+      </x:c>
+      <x:c r="B10" s="98" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>Trainers at Rank &gt;= Zone</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
+        <x:v>progression.zone_5.population_cap</x:v>
+      </x:c>
+      <x:c r="B11" s="98" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>Trainers</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>progression.zone_5.rank_count_gate</x:v>
+      </x:c>
+      <x:c r="B12" s="98" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>Trainers at Rank &gt;= Zone</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>progression.dormitory.upgrade_gold_base</x:v>
+      </x:c>
+      <x:c r="B13" s="98" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>Gold for level 2</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: cost unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>progression.town_hall.upgrade_gold_base</x:v>
+      </x:c>
+      <x:c r="B14" s="98" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>Gold for level 2</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: cost unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>progression.facility.upgrade_gold_base</x:v>
+      </x:c>
+      <x:c r="B15" s="98" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>Gold for level 2 or construction</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: generic facility cost unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>buildings.degraded.efficiency_multiplier</x:v>
+      </x:c>
+      <x:c r="B16" s="98" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2 and §1.6: maintenance deficit and damage reduce efficiency by half</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>buildings.generic.upkeep_per_level_per_day</x:v>
+      </x:c>
+      <x:c r="B17" s="98" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Gold/level/day</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.4: operating cost formula unspecified; src/Game.Domain/Config/SimConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>progression.dormitory.upgrade_cost_growth</x:v>
+      </x:c>
+      <x:c r="B18" s="98" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="str">
+        <x:v>multiplier per target level</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; §1.7 legacy curve needs recalculation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47" t="str">
+        <x:v>progression.facility_upgrade_minutes</x:v>
+      </x:c>
+      <x:c r="B19" s="98" t="n">
+        <x:v>2880</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E19" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: several days; exact duration unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47" t="str">
+        <x:v>progression.town_hall.max_level</x:v>
+      </x:c>
+      <x:c r="B20" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C20" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="47" t="str">
+        <x:v>progression.town_hall.levels_per_tier</x:v>
+      </x:c>
+      <x:c r="B21" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="str">
+        <x:v>levels/tier</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="47" t="str">
+        <x:v>progression.dormitory.max_level</x:v>
+      </x:c>
+      <x:c r="B22" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E22" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="47" t="str">
+        <x:v>progression.start_town_hall_level</x:v>
+      </x:c>
+      <x:c r="B23" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="47" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs: FTUE start default</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="47" t="str">
+        <x:v>progression.start_dormitory_level</x:v>
+      </x:c>
+      <x:c r="B24" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="47" t="str">
+        <x:v>src/Game.Domain/Config/SimConfig.cs: FTUE start default</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="47" t="str">
+        <x:v>progression.start_rebuilt_facility_level</x:v>
+      </x:c>
+      <x:c r="B25" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C25" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E25" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four defaults start rebuilt; start level unspecified; src/Game.Domain/Config/SimConfig.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="47" t="str">
+        <x:v>reputation.service_level_normalizer</x:v>
+      </x:c>
+      <x:c r="B26" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>building levels</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: relationship specified; scale is not</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="47" t="str">
+        <x:v>reputation.bankruptcy_penalty</x:v>
+      </x:c>
+      <x:c r="B27" s="98" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C27" s="47" t="str">
+        <x:v>points/bankruptcy</x:v>
+      </x:c>
+      <x:c r="D27" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E27" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: coefficient unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="47" t="str">
+        <x:v>reputation.traffic_base</x:v>
+      </x:c>
+      <x:c r="B28" s="98" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C28" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D28" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E28" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: mapping unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="47" t="str">
+        <x:v>reputation.traffic_per_point</x:v>
+      </x:c>
+      <x:c r="B29" s="98" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C29" s="47" t="str">
+        <x:v>multiplier/point</x:v>
+      </x:c>
+      <x:c r="D29" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E29" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: mapping unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="47" t="str">
+        <x:v>reputation.applicant_rarity_per_point</x:v>
+      </x:c>
+      <x:c r="B30" s="98" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C30" s="47" t="str">
+        <x:v>chance modifier/point</x:v>
+      </x:c>
+      <x:c r="D30" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E30" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: mapping unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="47" t="str">
+        <x:v>reputation.inspection_base</x:v>
+      </x:c>
+      <x:c r="B31" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C31" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D31" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E31" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: mapping unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="47" t="str">
+        <x:v>reputation.inspection_per_point</x:v>
+      </x:c>
+      <x:c r="B32" s="98" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="C32" s="47" t="str">
+        <x:v>multiplier/point</x:v>
+      </x:c>
+      <x:c r="D32" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E32" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §2.2: mapping unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="47" t="str">
+        <x:v>events.random_crisis.check_interval_minutes</x:v>
+      </x:c>
+      <x:c r="B33" s="98" t="n">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="C33" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D33" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E33" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B/1D: random event cadence unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="47" t="str">
+        <x:v>events.random_crisis.probability_per_check</x:v>
+      </x:c>
+      <x:c r="B34" s="98" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C34" s="47" t="str">
+        <x:v>probability/check</x:v>
+      </x:c>
+      <x:c r="D34" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E34" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B/1D: random event chance unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="47" t="str">
+        <x:v>events.black_friday.duration_days</x:v>
+      </x:c>
+      <x:c r="B35" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C35" s="47" t="str">
+        <x:v>in-game days</x:v>
+      </x:c>
+      <x:c r="D35" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E35" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="47" t="str">
+        <x:v>events.black_friday.impulse_units_per_product</x:v>
+      </x:c>
+      <x:c r="B36" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C36" s="47" t="str">
+        <x:v>units/Trainer/product</x:v>
+      </x:c>
+      <x:c r="D36" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E36" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1A: quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="47" t="str">
+        <x:v>events.labor_inspection.tax_threshold</x:v>
+      </x:c>
+      <x:c r="B37" s="98" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C37" s="47" t="str">
+        <x:v>fraction</x:v>
+      </x:c>
+      <x:c r="D37" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E37" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="47" t="str">
+        <x:v>events.labor_inspection.stress_threshold</x:v>
+      </x:c>
+      <x:c r="B38" s="98" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C38" s="47" t="str">
+        <x:v>stress points</x:v>
+      </x:c>
+      <x:c r="D38" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E38" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B; docs/designs/02_HUB_Economy_Infrastructure.md §2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="47" t="str">
+        <x:v>events.labor_inspection.fine_fraction</x:v>
+      </x:c>
+      <x:c r="B39" s="98" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C39" s="47" t="str">
+        <x:v>fraction of Treasury</x:v>
+      </x:c>
+      <x:c r="D39" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E39" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B: fine unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="47" t="str">
+        <x:v>events.labor_inspection.cooldown_minutes</x:v>
+      </x:c>
+      <x:c r="B40" s="98" t="n">
+        <x:v>43200</x:v>
+      </x:c>
+      <x:c r="C40" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D40" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E40" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B: cadence unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="47" t="str">
+        <x:v>events.labor_inspection.resolution_minutes</x:v>
+      </x:c>
+      <x:c r="B41" s="98" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C41" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D41" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E41" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1B: response window unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="47" t="str">
+        <x:v>events.breeding_season.duration_days</x:v>
+      </x:c>
+      <x:c r="B42" s="98" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C42" s="47" t="str">
+        <x:v>in-game days</x:v>
+      </x:c>
+      <x:c r="D42" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E42" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1C: duration unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="47" t="str">
+        <x:v>events.breeding_season.rare_iv_weight_multiplier</x:v>
+      </x:c>
+      <x:c r="B43" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C43" s="47" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D43" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E43" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1C: increase unquantified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="47" t="str">
+        <x:v>events.breeding_season.capture_goods_demand_multiplier</x:v>
+      </x:c>
+      <x:c r="B44" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C44" s="47" t="str">
+        <x:v>quantity multiplier</x:v>
+      </x:c>
+      <x:c r="D44" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E44" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1C: demand increase is unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="47" t="str">
+        <x:v>events.breeding_season.capture_goods_price_cap_multiplier</x:v>
+      </x:c>
+      <x:c r="B45" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C45" s="47" t="str">
+        <x:v>maximum price multiplier</x:v>
+      </x:c>
+      <x:c r="D45" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E45" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1C: Director may set price to 3x.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="47" t="str">
+        <x:v>events.monster_flu.duration_days</x:v>
+      </x:c>
+      <x:c r="B46" s="98" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C46" s="47" t="str">
+        <x:v>in-game days</x:v>
+      </x:c>
+      <x:c r="D46" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E46" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1D: duration unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="47" t="str">
+        <x:v>events.monster_flu.daily_hp_loss_fraction</x:v>
+      </x:c>
+      <x:c r="B47" s="98" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C47" s="47" t="str">
+        <x:v>fraction of max HP/day</x:v>
+      </x:c>
+      <x:c r="D47" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E47" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1D: ongoing HP loss rate unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="47" t="str">
+        <x:v>events.monster_flu.initial_hp_fraction</x:v>
+      </x:c>
+      <x:c r="B48" s="98" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C48" s="47" t="str">
+        <x:v>fraction of current HP</x:v>
+      </x:c>
+      <x:c r="D48" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E48" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1D: Monsters lose 50% HP at flu onset</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="47" t="str">
+        <x:v>events.monster_flu.vaccine_units_to_cure</x:v>
+      </x:c>
+      <x:c r="B49" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C49" s="47" t="str">
+        <x:v>vaccine units/outbreak</x:v>
+      </x:c>
+      <x:c r="D49" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E49" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1D: vaccine can cut the epidemic; usage quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="47" t="str">
+        <x:v>events.monster_flu.hospital_revenue_bonus_per_day</x:v>
+      </x:c>
+      <x:c r="B50" s="98" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C50" s="47" t="str">
+        <x:v>Gold/day</x:v>
+      </x:c>
+      <x:c r="D50" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E50" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1D: Hospital shares rise; revenue signal amount unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="47" t="str">
+        <x:v>events.breeding_season.ordinary_iv_weight</x:v>
+      </x:c>
+      <x:c r="B51" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C51" s="47" t="str">
+        <x:v>weight/grade</x:v>
+      </x:c>
+      <x:c r="D51" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E51" s="47" t="str">
+        <x:v>src/Game.Domain/Hub/HubWorld.Events.cs: equal ordinary-grade baseline; weighting model provisional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="47" t="str">
+        <x:v>events.breeding_season.rare_iv_grade_count</x:v>
+      </x:c>
+      <x:c r="B52" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C52" s="47" t="str">
+        <x:v>grades</x:v>
+      </x:c>
+      <x:c r="D52" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E52" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1C names rare IV grades S and SS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="47" t="str">
+        <x:v>events.siege.frequency</x:v>
+      </x:c>
+      <x:c r="B53" s="98" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="C53" s="47" t="str">
+        <x:v>events per period</x:v>
+      </x:c>
+      <x:c r="D53" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E53" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E; cadence unspecified; not implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="47" t="str">
+        <x:v>events.monster_siege.victory_gold</x:v>
+      </x:c>
+      <x:c r="B54" s="98" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C54" s="47" t="str">
+        <x:v>Gold/winning Trainer</x:v>
+      </x:c>
+      <x:c r="D54" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E54" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E; reward amount unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="47" t="str">
+        <x:v>events.monster_siege.boss_core_count</x:v>
+      </x:c>
+      <x:c r="B55" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C55" s="47" t="str">
+        <x:v>Boss Cores/winning Trainer</x:v>
+      </x:c>
+      <x:c r="D55" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E55" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §2: valuable Boss Core reward quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="47" t="str">
+        <x:v>events.world_boss.cooldown_minutes</x:v>
+      </x:c>
+      <x:c r="B56" s="98" t="n">
+        <x:v>43200</x:v>
+      </x:c>
+      <x:c r="C56" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D56" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E56" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25; exact cooldown unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="47" t="str">
+        <x:v>events.world_boss.activation_gold</x:v>
+      </x:c>
+      <x:c r="B57" s="98" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C57" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D57" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E57" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25; cost unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="47" t="str">
+        <x:v>buildings.facility_catalog_entries</x:v>
+      </x:c>
+      <x:c r="B58" s="98" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C58" s="47" t="str">
+        <x:v>facilities</x:v>
+      </x:c>
+      <x:c r="D58" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E58" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="47" t="str">
+        <x:v>buildings.level_25.max_level</x:v>
+      </x:c>
+      <x:c r="B59" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C59" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D59" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E59" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="47" t="str">
+        <x:v>buildings.level_5.max_level</x:v>
+      </x:c>
+      <x:c r="B60" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C60" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D60" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E60" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="47" t="str">
+        <x:v>buildings.level_1.max_level</x:v>
+      </x:c>
+      <x:c r="B61" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C61" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D61" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E61" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: Bounty Board is a prop</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="47" t="str">
+        <x:v>progression.construction.wood_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B62" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C62" s="47" t="str">
+        <x:v>Wood ingots/target level</x:v>
+      </x:c>
+      <x:c r="D62" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E62" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="47" t="str">
+        <x:v>progression.construction.stone_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B63" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C63" s="47" t="str">
+        <x:v>Stone ingots/target level</x:v>
+      </x:c>
+      <x:c r="D63" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E63" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: quantity unspecified; mapped to Ore Tier 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="47" t="str">
+        <x:v>progression.construction.iron_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B64" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C64" s="47" t="str">
+        <x:v>Iron ingots/target level</x:v>
+      </x:c>
+      <x:c r="D64" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E64" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2: quantity unspecified; mapped to Ore Tier 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="47" t="str">
+        <x:v>buildings.repair.gold_per_level</x:v>
+      </x:c>
+      <x:c r="B65" s="98" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C65" s="47" t="str">
+        <x:v>Gold/building level</x:v>
+      </x:c>
+      <x:c r="D65" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E65" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: repair cost scales with level; base unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="47" t="str">
+        <x:v>buildings.repair.minutes</x:v>
+      </x:c>
+      <x:c r="B66" s="98" t="n">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="C66" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D66" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E66" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: repair duration unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="47" t="str">
+        <x:v>buildings.repair.wood_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B67" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C67" s="47" t="str">
+        <x:v>Wood ingots/building level</x:v>
+      </x:c>
+      <x:c r="D67" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E67" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="47" t="str">
+        <x:v>buildings.repair.stone_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B68" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C68" s="47" t="str">
+        <x:v>Stone ingots/building level</x:v>
+      </x:c>
+      <x:c r="D68" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E68" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="47" t="str">
+        <x:v>buildings.repair.iron_ingots_per_level</x:v>
+      </x:c>
+      <x:c r="B69" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C69" s="47" t="str">
+        <x:v>Iron ingots/building level</x:v>
+      </x:c>
+      <x:c r="D69" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E69" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: quantity unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="47" t="str">
+        <x:v>events.monster_siege.duration_minutes</x:v>
+      </x:c>
+      <x:c r="B70" s="98" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="C70" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D70" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E70" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: duration unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="47" t="str">
+        <x:v>events.monster_siege.minimum_rank</x:v>
+      </x:c>
+      <x:c r="B71" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C71" s="47" t="str">
+        <x:v>Trainer rank</x:v>
+      </x:c>
+      <x:c r="D71" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E71" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: defender eligibility unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="47" t="str">
+        <x:v>events.monster_siege.enemy_hp</x:v>
+      </x:c>
+      <x:c r="B72" s="98" t="n">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="C72" s="47" t="str">
+        <x:v>HP</x:v>
+      </x:c>
+      <x:c r="D72" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E72" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: enemy scaling unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="47" t="str">
+        <x:v>events.monster_siege.enemy_attack</x:v>
+      </x:c>
+      <x:c r="B73" s="98" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C73" s="47" t="str">
+        <x:v>ATK</x:v>
+      </x:c>
+      <x:c r="D73" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E73" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: enemy scaling unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="47" t="str">
+        <x:v>events.monster_siege.enemy_defense</x:v>
+      </x:c>
+      <x:c r="B74" s="98" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C74" s="47" t="str">
+        <x:v>DEF</x:v>
+      </x:c>
+      <x:c r="D74" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E74" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: enemy scaling unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="47" t="str">
+        <x:v>events.monster_siege.enemy_attack_speed</x:v>
+      </x:c>
+      <x:c r="B75" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C75" s="47" t="str">
+        <x:v>attacks/round</x:v>
+      </x:c>
+      <x:c r="D75" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E75" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: enemy scaling unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="47" t="str">
+        <x:v>events.monster_siege.building_damage_probability</x:v>
+      </x:c>
+      <x:c r="B76" s="98" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="C76" s="47" t="str">
+        <x:v>probability on loss</x:v>
+      </x:c>
+      <x:c r="D76" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E76" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: chance unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="47" t="str">
+        <x:v>events.monster_siege.minimum_win_fraction</x:v>
+      </x:c>
+      <x:c r="B77" s="98" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C77" s="47" t="str">
+        <x:v>fraction</x:v>
+      </x:c>
+      <x:c r="D77" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E77" s="47" t="str">
+        <x:v>docs/designs/06_Events_PVE_PVP.md §1E: group victory rule unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="47" t="str">
+        <x:v>events.world_boss.duration_minutes</x:v>
+      </x:c>
+      <x:c r="B78" s="98" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="C78" s="47" t="str">
+        <x:v>in-game minutes</x:v>
+      </x:c>
+      <x:c r="D78" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E78" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: duration unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="47" t="str">
+        <x:v>events.world_boss.minimum_rank</x:v>
+      </x:c>
+      <x:c r="B79" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C79" s="47" t="str">
+        <x:v>Trainer rank</x:v>
+      </x:c>
+      <x:c r="D79" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E79" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: rank threshold unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="47" t="str">
+        <x:v>events.world_boss.hp</x:v>
+      </x:c>
+      <x:c r="B80" s="98" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C80" s="47" t="str">
+        <x:v>HP</x:v>
+      </x:c>
+      <x:c r="D80" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E80" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: Boss combat stats unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="47" t="str">
+        <x:v>events.world_boss.attack</x:v>
+      </x:c>
+      <x:c r="B81" s="98" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C81" s="47" t="str">
+        <x:v>ATK</x:v>
+      </x:c>
+      <x:c r="D81" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E81" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: Boss combat stats unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="47" t="str">
+        <x:v>events.world_boss.defense</x:v>
+      </x:c>
+      <x:c r="B82" s="98" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C82" s="47" t="str">
+        <x:v>DEF</x:v>
+      </x:c>
+      <x:c r="D82" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E82" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: Boss combat stats unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="47" t="str">
+        <x:v>events.world_boss.attack_speed</x:v>
+      </x:c>
+      <x:c r="B83" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C83" s="47" t="str">
+        <x:v>attacks/round</x:v>
+      </x:c>
+      <x:c r="D83" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E83" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: Boss combat stats unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="47" t="str">
+        <x:v>events.world_boss.building_damage_probability</x:v>
+      </x:c>
+      <x:c r="B84" s="98" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="C84" s="47" t="str">
+        <x:v>probability on loss</x:v>
+      </x:c>
+      <x:c r="D84" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E84" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.6: chance unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="47" t="str">
+        <x:v>events.world_boss.crystal_count</x:v>
+      </x:c>
+      <x:c r="B85" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C85" s="47" t="str">
+        <x:v>crystals/winning Trainer</x:v>
+      </x:c>
+      <x:c r="D85" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E85" s="47" t="str">
+        <x:v>docs/designs/01_World_Map_Environment.md §25: quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="47" t="str">
+        <x:v>buildings.facility.town_hall.max_level</x:v>
+      </x:c>
+      <x:c r="B86" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C86" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D86" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E86" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="47" t="str">
+        <x:v>buildings.facility.town_hall.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B87" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C87" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D87" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E87" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="47" t="str">
+        <x:v>buildings.facility.town_hall.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B88" s="166" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C88" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D88" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E88" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="47" t="str">
+        <x:v>buildings.facility.town_hall.start_level</x:v>
+      </x:c>
+      <x:c r="B89" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C89" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D89" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E89" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: starts rebuilt; start level unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="47" t="str">
+        <x:v>buildings.facility.dormitory.max_level</x:v>
+      </x:c>
+      <x:c r="B90" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C90" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D90" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E90" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="47" t="str">
+        <x:v>buildings.facility.dormitory.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B91" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C91" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D91" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E91" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="47" t="str">
+        <x:v>buildings.facility.dormitory.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B92" s="166" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C92" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D92" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E92" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="47" t="str">
+        <x:v>buildings.facility.dormitory.start_level</x:v>
+      </x:c>
+      <x:c r="B93" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C93" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D93" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E93" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: starts rebuilt; start level unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="47" t="str">
+        <x:v>buildings.facility.trading_station.max_level</x:v>
+      </x:c>
+      <x:c r="B94" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C94" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D94" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E94" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="47" t="str">
+        <x:v>buildings.facility.trading_station.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B95" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C95" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D95" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E95" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="47" t="str">
+        <x:v>buildings.facility.trading_station.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B96" s="166" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C96" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D96" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E96" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="47" t="str">
+        <x:v>buildings.facility.trading_station.start_level</x:v>
+      </x:c>
+      <x:c r="B97" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C97" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D97" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E97" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: starts rebuilt; start level unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="47" t="str">
+        <x:v>buildings.facility.veterinary_hospital.max_level</x:v>
+      </x:c>
+      <x:c r="B98" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C98" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D98" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E98" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="47" t="str">
+        <x:v>buildings.facility.veterinary_hospital.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B99" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C99" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D99" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E99" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="47" t="str">
+        <x:v>buildings.facility.veterinary_hospital.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B100" s="166" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C100" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D100" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E100" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="47" t="str">
+        <x:v>buildings.facility.veterinary_hospital.start_level</x:v>
+      </x:c>
+      <x:c r="B101" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C101" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D101" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E101" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: starts rebuilt; start level unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="47" t="str">
+        <x:v>buildings.facility.inn.max_level</x:v>
+      </x:c>
+      <x:c r="B102" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C102" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D102" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E102" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="47" t="str">
+        <x:v>buildings.facility.inn.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B103" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C103" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D103" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E103" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="47" t="str">
+        <x:v>buildings.facility.inn.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B104" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C104" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D104" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E104" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="47" t="str">
+        <x:v>buildings.facility.inn.start_level</x:v>
+      </x:c>
+      <x:c r="B105" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C105" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D105" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E105" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="47" t="str">
+        <x:v>buildings.facility.restaurant.max_level</x:v>
+      </x:c>
+      <x:c r="B106" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C106" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D106" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E106" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="47" t="str">
+        <x:v>buildings.facility.restaurant.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B107" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C107" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D107" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E107" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="47" t="str">
+        <x:v>buildings.facility.restaurant.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B108" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C108" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D108" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E108" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="47" t="str">
+        <x:v>buildings.facility.restaurant.start_level</x:v>
+      </x:c>
+      <x:c r="B109" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C109" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D109" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E109" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="47" t="str">
+        <x:v>buildings.facility.refinery.max_level</x:v>
+      </x:c>
+      <x:c r="B110" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C110" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D110" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E110" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="47" t="str">
+        <x:v>buildings.facility.refinery.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B111" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C111" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D111" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E111" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="47" t="str">
+        <x:v>buildings.facility.refinery.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B112" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C112" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D112" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E112" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="47" t="str">
+        <x:v>buildings.facility.refinery.start_level</x:v>
+      </x:c>
+      <x:c r="B113" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C113" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D113" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E113" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="47" t="str">
+        <x:v>buildings.facility.tool_workshop.max_level</x:v>
+      </x:c>
+      <x:c r="B114" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C114" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D114" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E114" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="47" t="str">
+        <x:v>buildings.facility.tool_workshop.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B115" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C115" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D115" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E115" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="47" t="str">
+        <x:v>buildings.facility.tool_workshop.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B116" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C116" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D116" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E116" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="47" t="str">
+        <x:v>buildings.facility.tool_workshop.start_level</x:v>
+      </x:c>
+      <x:c r="B117" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C117" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D117" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E117" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="47" t="str">
+        <x:v>buildings.facility.bar.max_level</x:v>
+      </x:c>
+      <x:c r="B118" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C118" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D118" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E118" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="47" t="str">
+        <x:v>buildings.facility.bar.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B119" s="98" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C119" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D119" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E119" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="47" t="str">
+        <x:v>buildings.facility.bar.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B120" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C120" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D120" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E120" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="47" t="str">
+        <x:v>buildings.facility.bar.start_level</x:v>
+      </x:c>
+      <x:c r="B121" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C121" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D121" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E121" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="47" t="str">
+        <x:v>buildings.facility.monster_forge.max_level</x:v>
+      </x:c>
+      <x:c r="B122" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C122" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D122" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E122" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="47" t="str">
+        <x:v>buildings.facility.monster_forge.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B123" s="98" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C123" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D123" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E123" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="47" t="str">
+        <x:v>buildings.facility.monster_forge.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B124" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C124" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D124" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E124" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="47" t="str">
+        <x:v>buildings.facility.monster_forge.start_level</x:v>
+      </x:c>
+      <x:c r="B125" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C125" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D125" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E125" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="47" t="str">
+        <x:v>buildings.facility.textile_workshop.max_level</x:v>
+      </x:c>
+      <x:c r="B126" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C126" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D126" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E126" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="47" t="str">
+        <x:v>buildings.facility.textile_workshop.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B127" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C127" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D127" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E127" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="47" t="str">
+        <x:v>buildings.facility.textile_workshop.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B128" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C128" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D128" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E128" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="47" t="str">
+        <x:v>buildings.facility.textile_workshop.start_level</x:v>
+      </x:c>
+      <x:c r="B129" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C129" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D129" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E129" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="47" t="str">
+        <x:v>buildings.facility.bounty_board.max_level</x:v>
+      </x:c>
+      <x:c r="B130" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C130" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D130" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E130" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="47" t="str">
+        <x:v>buildings.facility.bounty_board.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B131" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C131" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D131" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E131" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 facility unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="47" t="str">
+        <x:v>buildings.facility.bounty_board.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B132" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C132" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D132" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E132" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="47" t="str">
+        <x:v>buildings.facility.bounty_board.start_level</x:v>
+      </x:c>
+      <x:c r="B133" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C133" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D133" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E133" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="47" t="str">
+        <x:v>buildings.facility.reactor.max_level</x:v>
+      </x:c>
+      <x:c r="B134" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C134" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D134" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E134" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="47" t="str">
+        <x:v>buildings.facility.reactor.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B135" s="98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C135" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D135" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E135" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="47" t="str">
+        <x:v>buildings.facility.reactor.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B136" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C136" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D136" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E136" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="47" t="str">
+        <x:v>buildings.facility.reactor.start_level</x:v>
+      </x:c>
+      <x:c r="B137" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C137" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D137" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E137" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="47" t="str">
+        <x:v>buildings.facility.reactor.required_zone</x:v>
+      </x:c>
+      <x:c r="B138" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C138" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D138" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E138" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="47" t="str">
+        <x:v>buildings.facility.warp_gate.max_level</x:v>
+      </x:c>
+      <x:c r="B139" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C139" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D139" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E139" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="47" t="str">
+        <x:v>buildings.facility.warp_gate.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B140" s="98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C140" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D140" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E140" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="47" t="str">
+        <x:v>buildings.facility.warp_gate.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B141" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C141" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D141" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E141" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="47" t="str">
+        <x:v>buildings.facility.warp_gate.start_level</x:v>
+      </x:c>
+      <x:c r="B142" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C142" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D142" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E142" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="47" t="str">
+        <x:v>buildings.facility.warp_gate.required_zone</x:v>
+      </x:c>
+      <x:c r="B143" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C143" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D143" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E143" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="47" t="str">
+        <x:v>buildings.facility.soda_factory.max_level</x:v>
+      </x:c>
+      <x:c r="B144" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C144" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D144" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E144" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="47" t="str">
+        <x:v>buildings.facility.soda_factory.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B145" s="98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C145" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D145" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E145" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="47" t="str">
+        <x:v>buildings.facility.soda_factory.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B146" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C146" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D146" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E146" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="47" t="str">
+        <x:v>buildings.facility.soda_factory.start_level</x:v>
+      </x:c>
+      <x:c r="B147" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C147" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D147" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E147" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="47" t="str">
+        <x:v>buildings.facility.soda_factory.required_zone</x:v>
+      </x:c>
+      <x:c r="B148" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C148" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D148" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E148" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="47" t="str">
+        <x:v>buildings.facility.general_store.max_level</x:v>
+      </x:c>
+      <x:c r="B149" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C149" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D149" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E149" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="47" t="str">
+        <x:v>buildings.facility.general_store.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B150" s="98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C150" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D150" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E150" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="47" t="str">
+        <x:v>buildings.facility.general_store.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B151" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C151" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D151" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E151" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="47" t="str">
+        <x:v>buildings.facility.general_store.start_level</x:v>
+      </x:c>
+      <x:c r="B152" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C152" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D152" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E152" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="47" t="str">
+        <x:v>buildings.facility.general_store.required_zone</x:v>
+      </x:c>
+      <x:c r="B153" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C153" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D153" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E153" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="47" t="str">
+        <x:v>buildings.facility.gene_bank.max_level</x:v>
+      </x:c>
+      <x:c r="B154" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C154" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D154" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E154" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="47" t="str">
+        <x:v>buildings.facility.gene_bank.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B155" s="98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C155" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D155" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E155" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="47" t="str">
+        <x:v>buildings.facility.gene_bank.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B156" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C156" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D156" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E156" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="47" t="str">
+        <x:v>buildings.facility.gene_bank.start_level</x:v>
+      </x:c>
+      <x:c r="B157" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C157" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D157" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E157" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="47" t="str">
+        <x:v>buildings.facility.gene_bank.required_zone</x:v>
+      </x:c>
+      <x:c r="B158" s="98" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C158" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D158" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E158" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="47" t="str">
+        <x:v>buildings.facility.jeweler.max_level</x:v>
+      </x:c>
+      <x:c r="B159" s="98" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C159" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D159" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E159" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="47" t="str">
+        <x:v>buildings.facility.jeweler.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B160" s="98" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C160" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D160" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E160" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="47" t="str">
+        <x:v>buildings.facility.jeweler.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B161" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C161" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D161" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E161" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="47" t="str">
+        <x:v>buildings.facility.jeweler.start_level</x:v>
+      </x:c>
+      <x:c r="B162" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C162" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D162" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E162" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="47" t="str">
+        <x:v>buildings.facility.jeweler.required_zone</x:v>
+      </x:c>
+      <x:c r="B163" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C163" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D163" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E163" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="47" t="str">
+        <x:v>buildings.facility.evolution_lab.max_level</x:v>
+      </x:c>
+      <x:c r="B164" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C164" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D164" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E164" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="47" t="str">
+        <x:v>buildings.facility.evolution_lab.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B165" s="98" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C165" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D165" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E165" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="47" t="str">
+        <x:v>buildings.facility.evolution_lab.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B166" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C166" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D166" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E166" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="47" t="str">
+        <x:v>buildings.facility.evolution_lab.start_level</x:v>
+      </x:c>
+      <x:c r="B167" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C167" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D167" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E167" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="47" t="str">
+        <x:v>buildings.facility.evolution_lab.required_zone</x:v>
+      </x:c>
+      <x:c r="B168" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C168" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D168" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E168" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="47" t="str">
+        <x:v>buildings.facility.academy.max_level</x:v>
+      </x:c>
+      <x:c r="B169" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C169" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D169" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E169" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="47" t="str">
+        <x:v>buildings.facility.academy.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B170" s="98" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C170" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D170" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E170" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="47" t="str">
+        <x:v>buildings.facility.academy.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B171" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C171" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D171" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E171" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="47" t="str">
+        <x:v>buildings.facility.academy.start_level</x:v>
+      </x:c>
+      <x:c r="B172" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C172" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D172" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E172" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="47" t="str">
+        <x:v>buildings.facility.academy.required_zone</x:v>
+      </x:c>
+      <x:c r="B173" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C173" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D173" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E173" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="47" t="str">
+        <x:v>buildings.facility.stock_exchange.max_level</x:v>
+      </x:c>
+      <x:c r="B174" s="98" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C174" s="47" t="str">
+        <x:v>levels</x:v>
+      </x:c>
+      <x:c r="D174" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E174" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="47" t="str">
+        <x:v>buildings.facility.stock_exchange.town_hall_unlock_level</x:v>
+      </x:c>
+      <x:c r="B175" s="98" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C175" s="47" t="str">
+        <x:v>Town Hall level</x:v>
+      </x:c>
+      <x:c r="D175" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E175" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1 tier unlock table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="47" t="str">
+        <x:v>buildings.facility.stock_exchange.starts_rebuilt</x:v>
+      </x:c>
+      <x:c r="B176" s="166" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C176" s="47" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D176" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E176" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: four facilities start ruined/rebuilt; others are built new</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="47" t="str">
+        <x:v>buildings.facility.stock_exchange.start_level</x:v>
+      </x:c>
+      <x:c r="B177" s="98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C177" s="47" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="D177" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E177" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: built new; starts unbuilt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="47" t="str">
+        <x:v>buildings.facility.stock_exchange.required_zone</x:v>
+      </x:c>
+      <x:c r="B178" s="98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C178" s="47" t="str">
+        <x:v>Zone</x:v>
+      </x:c>
+      <x:c r="D178" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E178" s="47" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -24009,6 +27449,93 @@
         <x:v>GDD 12 §1-2; docs/designs/02_HUB_Economy_Infrastructure.md §1.0; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>refinery_wood_ingot</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>Tinh chế Gỗ thành Phôi Gỗ</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>wood_tier_1</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Gỗ Tier 1</x:v>
+      </x:c>
+      <x:c r="F80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>refinery_stone_ingot</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Tinh chế Quặng Tier 1 thành Phôi Đá</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>ore_tier_1</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>Khoáng Tier 1</x:v>
+      </x:c>
+      <x:c r="F81" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>refinery_iron_ingot</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Tinh chế Quặng Tier 2 thành Phôi Sắt</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>ore_tier_2</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>Khoáng Tier 2</x:v>
+      </x:c>
+      <x:c r="F82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -26194,26 +29721,91 @@
       </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="27"/>
-      <x:c r="B78" s="27"/>
-      <x:c r="C78" s="27"/>
-      <x:c r="D78" s="27"/>
-      <x:c r="E78" s="27"/>
-      <x:c r="F78" s="27"/>
-      <x:c r="G78" s="27"/>
-      <x:c r="H78" s="27"/>
-      <x:c r="I78" s="27"/>
+      <x:c r="A78" s="27" t="str">
+        <x:v>refinery_wood_ingot</x:v>
+      </x:c>
+      <x:c r="B78" s="27" t="str">
+        <x:v>Tinh chế Gỗ thành Phôi Gỗ</x:v>
+      </x:c>
+      <x:c r="C78" s="27" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D78" s="27" t="str">
+        <x:v>wood_ingot</x:v>
+      </x:c>
+      <x:c r="E78" s="27" t="str">
+        <x:v>Phôi Gỗ</x:v>
+      </x:c>
+      <x:c r="F78" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G78" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H78" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I78" s="27" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="27"/>
-      <x:c r="B79" s="27"/>
-      <x:c r="C79" s="27"/>
-      <x:c r="D79" s="27"/>
-      <x:c r="E79" s="27"/>
-      <x:c r="F79" s="27"/>
-      <x:c r="G79" s="27"/>
-      <x:c r="H79" s="27"/>
-      <x:c r="I79" s="27"/>
+      <x:c r="A79" s="27" t="str">
+        <x:v>refinery_stone_ingot</x:v>
+      </x:c>
+      <x:c r="B79" s="27" t="str">
+        <x:v>Tinh chế Quặng Tier 1 thành Phôi Đá</x:v>
+      </x:c>
+      <x:c r="C79" s="27" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D79" s="27" t="str">
+        <x:v>stone_ingot</x:v>
+      </x:c>
+      <x:c r="E79" s="27" t="str">
+        <x:v>Phôi Đá</x:v>
+      </x:c>
+      <x:c r="F79" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G79" s="27" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H79" s="27" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I79" s="27" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>refinery_iron_ingot</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>Tinh chế Quặng Tier 2 thành Phôi Sắt</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>refinery</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>iron_ingot</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Phôi Sắt</x:v>
+      </x:c>
+      <x:c r="F80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>đơn vị</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.2; src/Game.Domain/Materials/MaterialCatalog.cs</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(domain): complete quests and KPI sub-project
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,26 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R10789b43e96948e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R59a974accfaf4b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Re260193becfc463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R7fd798922ae34acc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Rbbc0f1b7b1dd4a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rf86d881f8a6e44ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R6a7f9ba2aaed4612"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R7885bf1965554c29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="Rd582fe2f35e948b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="Rdefc22f573124f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R428c4efb8bed4ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R133cc75eee1f412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Refd1053fecba4a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R7a9814b8647b4fdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Rd07e849ca9c44737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R13684d74a9b34650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R4cd1090cdf6743d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="R2245c98daa2d4789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="Rb9995bbfcb994fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP6 Progression &amp; Events" sheetId="20" r:id="Rb98afae9c0854aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59c2a02009c74b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R09cb464f54a0473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rcbe36715bb6c4a94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rf3fcb08481e6427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Re8cdec4f13fc4e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rffaa75cc247347b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R9dd0e255a26c4192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R352d511ec8064138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R0127f764f9ff4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R5c8b0518ade0487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R43cc549be42c47d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R8683893c510b4083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Rc9f9d9f87ecc4236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="Rb5fb04268a3f4160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="R862b5d0d9e7f4bdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="Ra158789ec6d74ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R75f8620d253a4343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="Rf096e2686d274282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="R3faf53822a8e424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP6 Progression &amp; Events" sheetId="20" r:id="Rd5fa2543af1b4a10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest &amp; KPI" sheetId="21" r:id="R3480a00717f3474f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -118,12 +119,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="28">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -283,7 +294,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="174">
+  <x:cellXfs count="188">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -686,6 +697,36 @@
     <x:xf numFmtId="0" fontId="3" fillId="27" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1074,6 +1115,14 @@
         <x:v>See SP6 Progression &amp; Events sheet; all parameters carry status and source.</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>Quest &amp; KPI</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Campaign and Daily/Weekly KPI balance assumptions; statuses and sources included.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15871,6 +15920,459 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="183" t="str">
+        <x:v>Early Access · Quest &amp; KPI</x:v>
+      </x:c>
+      <x:c r="B1" s="183"/>
+      <x:c r="C1" s="183"/>
+      <x:c r="D1" s="183"/>
+      <x:c r="E1" s="183"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="187" t="str">
+        <x:v>Stable ID</x:v>
+      </x:c>
+      <x:c r="B2" s="187" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C2" s="187" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="D2" s="187" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E2" s="187" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>quest.campaign.exploit_foundation.requirements</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>requirements/quest</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: Zone 2 and Veterinary Hospital level 2 are conjunctive requirements</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>quest.campaign.exploit_foundation.zone_number</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>zone number</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: Nền Móng Bóc Lột requires Zone 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>quest.campaign.exploit_foundation.hospital_level</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>facility level</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: Nền Móng Bóc Lột requires Veterinary Hospital level 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>quest.campaign.new_class.requirements</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>requirements/quest</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: Giai Cấp Mới requires Epic Trainer recruitment; content awaits recruitment support</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>quest.daily.medicine_gold_target</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>Gold/day</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1B; docs/designs/13_Balance_Parameters.md §7: GDD example target is a placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>quest.daily.stock_operations</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>settled director stock operations/day</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1B; docs/designs/13_Balance_Parameters.md §7: GDD example target is a placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>quest.daily.liquor_units</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>units/day</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1B; docs/designs/13_Balance_Parameters.md §7: GDD example target is a placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>quest.weekly.gene_confiscations</x:v>
+      </x:c>
+      <x:c r="B10" s="47" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>monsters/week</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1B; docs/designs/13_Balance_Parameters.md §7: GDD example target is a placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
+        <x:v>quest.weekly.protection_charm_units</x:v>
+      </x:c>
+      <x:c r="B11" s="47" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>units/week</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1B; docs/designs/13_Balance_Parameters.md §7: GDD example target is a placeholder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>quest.daily.period_days</x:v>
+      </x:c>
+      <x:c r="B12" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>in-game days</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: daily reset cadence; absolute time anchor is a simulator convention</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>quest.weekly.period_days</x:v>
+      </x:c>
+      <x:c r="B13" s="47" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>in-game days</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: weekly reset cadence; seven-day length and epoch anchor are simulator conventions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>quest.reward.daily.gold</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: sponsor reward required; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>quest.reward.daily.gems</x:v>
+      </x:c>
+      <x:c r="B15" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>Gems</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: reward may include Gem; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>quest.reward.weekly.gold</x:v>
+      </x:c>
+      <x:c r="B16" s="47" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: sponsor reward required; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>quest.reward.weekly.gems</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Gems</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1: reward may include Gem; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>quest.reward.campaign.gold</x:v>
+      </x:c>
+      <x:c r="B18" s="47" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: sponsor reward required; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47" t="str">
+        <x:v>quest.reward.campaign.gems</x:v>
+      </x:c>
+      <x:c r="B19" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="str">
+        <x:v>Gems</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E19" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: reward may include Gem; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47" t="str">
+        <x:v>quest.reward.campaign.building_permits</x:v>
+      </x:c>
+      <x:c r="B20" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="47" t="str">
+        <x:v>permits</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E20" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: building permits are a reward; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="47" t="str">
+        <x:v>quest.reward.campaign.high_tier_invitations</x:v>
+      </x:c>
+      <x:c r="B21" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="str">
+        <x:v>invitations</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E21" s="47" t="str">
+        <x:v>docs/designs/08_Quests_Achievements_Collections.md §1A: high-tier invitations are a reward; quantity unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="47" t="str">
+        <x:v>quest.reward.campaign.protection_charms</x:v>
+      </x:c>
+      <x:c r="B22" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="str">
+        <x:v>Protection Charms</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E22" s="47" t="str">
+        <x:v>docs/designs/07_Monetization_Model.md: Main Quest provides free Protection Charms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="47" t="str">
+        <x:v>quest.reward.weekly.protection_charms</x:v>
+      </x:c>
+      <x:c r="B23" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="str">
+        <x:v>Protection Charms</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E23" s="47" t="str">
+        <x:v>docs/designs/07_Monetization_Model.md: weekly KPI provides free Protection Charms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="47" t="str">
+        <x:v>quest.protection_charm.offer_price</x:v>
+      </x:c>
+      <x:c r="B24" s="47" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>Gold/Charm</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E24" s="47" t="str">
+        <x:v>docs/designs/07_Monetization_Model.md: Director sets Trainer sale price; default matches product.price.protection_charm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="47" t="str">
+        <x:v>quest.protection_charm.expected_avoided_loss</x:v>
+      </x:c>
+      <x:c r="B25" s="47" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C25" s="47" t="str">
+        <x:v>Gold</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E25" s="47" t="str">
+        <x:v>docs/designs/07_Monetization_Model.md: AI buys below expected enhancement loss; expected value unspecified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="47" t="str">
+        <x:v>quest.protection_charm.maximum_fulfillment</x:v>
+      </x:c>
+      <x:c r="B26" s="47" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>Charms/call</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E26" s="47" t="str">
+        <x:v>Provider/reward fulfillment bound for deterministic simulation; GDD gives no stock batch limit</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
fix: close remaining domain GDD behavior gaps
</commit_message>
<xml_diff>
--- a/docs/balance/MonsterHUB_Balance.xlsx
+++ b/docs/balance/MonsterHUB_Balance.xlsx
@@ -2,27 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59c2a02009c74b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R09cb464f54a0473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rcbe36715bb6c4a94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="Rf3fcb08481e6427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="Re8cdec4f13fc4e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rffaa75cc247347b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="R9dd0e255a26c4192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="R352d511ec8064138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R0127f764f9ff4a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R5c8b0518ade0487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R43cc549be42c47d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R8683893c510b4083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="Rc9f9d9f87ecc4236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="Rb5fb04268a3f4160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="R862b5d0d9e7f4bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="Ra158789ec6d74ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="R75f8620d253a4343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="Rf096e2686d274282"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="R3faf53822a8e424b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP6 Progression &amp; Events" sheetId="20" r:id="Rd5fa2543af1b4a10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest &amp; KPI" sheetId="21" r:id="R3480a00717f3474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4131a2ba00024d8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R8221ada922864a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Config" sheetId="3" r:id="Rd98051bc041c433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buildings" sheetId="4" r:id="R1e213ec443a140c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="5" r:id="R7e696e9d9db148e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Catalog" sheetId="6" r:id="Rb45edd9a33534838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Inputs" sheetId="7" r:id="Reb02e4a71882441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recipe Outputs" sheetId="8" r:id="Rb7c1fd69ff044996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merchant" sheetId="9" r:id="R70cd691075dc4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Controls" sheetId="10" r:id="R04b5150459344f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="11" r:id="R325efa5c98544276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Workshops" sheetId="12" r:id="R53486a9298574f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stalls" sheetId="13" r:id="R5bb5c60f12574e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Catalog" sheetId="14" r:id="R9352c82b8571432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat &amp; Capture" sheetId="15" r:id="Ra57f57a5ac8a4017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones &amp; Loot" sheetId="16" r:id="R4cbd6ea9e0864b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster Lifecycle" sheetId="17" r:id="Rad2326359d744091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear &amp; Durability" sheetId="18" r:id="Rd451326092e04d58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="19" r:id="R342c4cf2993046d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP6 Progression &amp; Events" sheetId="20" r:id="R750a77818e264b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest &amp; KPI" sheetId="21" r:id="R4b9d33b3a57b47a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15912,6 +15912,23 @@
         <x:v>docs/designs/02_HUB_Economy_Infrastructure.md §1.1: tier requires corresponding Zone</x:v>
       </x:c>
     </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="4" t="str">
+        <x:v>events.black_friday.junk_gear_price</x:v>
+      </x:c>
+      <x:c r="B179" s="4" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C179" s="4" t="str">
+        <x:v>Gold/gear item</x:v>
+      </x:c>
+      <x:c r="D179" s="4" t="str">
+        <x:v>Prototype</x:v>
+      </x:c>
+      <x:c r="E179" s="4" t="str">
+        <x:v>docs/designs/05 §1 and docs/designs/06 §1A: impulse gear purchase is specified, price is not; runtime default in HubEventConfig.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>

</xml_diff>